<commit_message>
Dashboard update 2026-08-08 11:06
</commit_message>
<xml_diff>
--- a/excel/Crowdpear.xlsx
+++ b/excel/Crowdpear.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="27932"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="30228"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\evald\OneDrive\Dokumentai\portfolio-analytics\portfolio-v2\excel\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Investavimas 2026.06.03\Crowdpear\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{34883093-1794-4D37-985D-5F9AA8E5449C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8B5D66E7-71A4-426B-A863-4C7DDD7F5D2C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" firstSheet="19" activeTab="27" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="17520" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Overview" sheetId="1" r:id="rId1"/>
@@ -429,18 +429,12 @@
       <scheme val="minor"/>
     </font>
   </fonts>
-  <fills count="3">
+  <fills count="2">
     <fill>
       <patternFill patternType="none"/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFFFFF00"/>
-        <bgColor indexed="64"/>
-      </patternFill>
     </fill>
   </fills>
   <borders count="7">
@@ -534,7 +528,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="37">
+  <cellXfs count="36">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center"/>
@@ -607,12 +601,6 @@
     <xf numFmtId="2" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="165" fontId="0" fillId="2" borderId="1" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
@@ -633,6 +621,9 @@
     </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="165" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="2">
@@ -3128,39 +3119,39 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:29" x14ac:dyDescent="0.25">
-      <c r="A1" s="30" t="s">
-        <v>0</v>
-      </c>
-      <c r="B1" s="31"/>
-      <c r="C1" s="31"/>
-      <c r="D1" s="31"/>
-      <c r="E1" s="31"/>
-      <c r="F1" s="31"/>
-      <c r="G1" s="32"/>
-      <c r="H1" s="33" t="s">
+      <c r="A1" s="28" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="29"/>
+      <c r="C1" s="29"/>
+      <c r="D1" s="29"/>
+      <c r="E1" s="29"/>
+      <c r="F1" s="29"/>
+      <c r="G1" s="30"/>
+      <c r="H1" s="31" t="s">
         <v>88</v>
       </c>
-      <c r="I1" s="33"/>
-      <c r="J1" s="33"/>
-      <c r="K1" s="33"/>
-      <c r="L1" s="33"/>
-      <c r="M1" s="33"/>
-      <c r="O1" s="33" t="s">
+      <c r="I1" s="31"/>
+      <c r="J1" s="31"/>
+      <c r="K1" s="31"/>
+      <c r="L1" s="31"/>
+      <c r="M1" s="31"/>
+      <c r="O1" s="31" t="s">
         <v>92</v>
       </c>
-      <c r="P1" s="33"/>
-      <c r="Q1" s="33"/>
-      <c r="R1" s="33"/>
-      <c r="S1" s="34" t="s">
+      <c r="P1" s="31"/>
+      <c r="Q1" s="31"/>
+      <c r="R1" s="31"/>
+      <c r="S1" s="32" t="s">
         <v>45</v>
       </c>
-      <c r="T1" s="34"/>
-      <c r="U1" s="34" t="s">
+      <c r="T1" s="32"/>
+      <c r="U1" s="32" t="s">
         <v>38</v>
       </c>
-      <c r="V1" s="34"/>
-      <c r="W1" s="34"/>
-      <c r="X1" s="34"/>
+      <c r="V1" s="32"/>
+      <c r="W1" s="32"/>
+      <c r="X1" s="32"/>
     </row>
     <row r="2" spans="1:29" x14ac:dyDescent="0.25">
       <c r="A2" s="6" t="s">
@@ -3326,7 +3317,7 @@
       </c>
       <c r="X3" s="14">
         <f ca="1">XIRR(Pinigai!K2:K200,Pinigai!A2:A200)</f>
-        <v>0.13074142336845396</v>
+        <v>0.12784344553947447</v>
       </c>
       <c r="AC3" s="4" t="str">
         <f ca="1">'Užnerio butai III'!AA2</f>
@@ -3827,7 +3818,7 @@
       </c>
       <c r="J12" s="10">
         <f ca="1">'Sfintii Arhangheli 21'!B13</f>
-        <v>42</v>
+        <v>33</v>
       </c>
       <c r="K12" s="10" t="str">
         <f ca="1">'Sfintii Arhangheli 21'!S3</f>
@@ -3941,7 +3932,7 @@
       </c>
       <c r="J14" s="10">
         <f ca="1">'Vienbutis Minsko 5A'!B13</f>
-        <v>49</v>
+        <v>40</v>
       </c>
       <c r="K14" s="10" t="str">
         <f ca="1">'Vienbutis Minsko 5A'!S3</f>
@@ -4055,7 +4046,7 @@
       </c>
       <c r="J16" s="10">
         <f ca="1">'Miškininkų 30 II'!B13</f>
-        <v>100</v>
+        <v>91</v>
       </c>
       <c r="K16" s="10" t="str">
         <f ca="1">'Miškininkų 30 II'!S3</f>
@@ -4112,7 +4103,7 @@
       </c>
       <c r="J17" s="10">
         <f ca="1">'Sūduvos 8-2'!B13</f>
-        <v>139</v>
+        <v>130</v>
       </c>
       <c r="K17" s="10" t="str">
         <f ca="1">'Sūduvos 8-2'!S3</f>
@@ -4169,7 +4160,7 @@
       </c>
       <c r="J18" s="10">
         <f ca="1">'Birelių namas II'!B13</f>
-        <v>146</v>
+        <v>137</v>
       </c>
       <c r="K18" s="10" t="str">
         <f ca="1">'Birelių namas II'!S3</f>
@@ -4283,7 +4274,7 @@
       </c>
       <c r="J20" s="10">
         <f ca="1">'Vingio namai XIV'!B13</f>
-        <v>188</v>
+        <v>179</v>
       </c>
       <c r="K20" s="10" t="str">
         <f ca="1">'Vingio namai XIV'!S3</f>
@@ -4397,7 +4388,7 @@
       </c>
       <c r="J22" s="10">
         <f ca="1">'Namas Panevėžyje'!B13</f>
-        <v>114</v>
+        <v>105</v>
       </c>
       <c r="K22" s="10" t="str">
         <f ca="1">'Namas Panevėžyje'!S3</f>
@@ -4511,11 +4502,11 @@
       </c>
       <c r="J24" s="10">
         <f ca="1">'Horizonto 2A XII'!B13</f>
-        <v>133</v>
+        <v>124</v>
       </c>
       <c r="K24" s="10">
         <f ca="1">'Horizonto 2A XII'!S3</f>
-        <v>29</v>
+        <v>38</v>
       </c>
       <c r="L24" s="4">
         <f>'Horizonto 2A XII'!N3</f>
@@ -4568,7 +4559,7 @@
       </c>
       <c r="J25" s="10">
         <f ca="1">'Tautvilo kotedžai XIV'!B13</f>
-        <v>317</v>
+        <v>308</v>
       </c>
       <c r="K25" s="10" t="str">
         <f ca="1">'Tautvilo kotedžai XIV'!S3</f>
@@ -4625,7 +4616,7 @@
       </c>
       <c r="J26" s="10">
         <f ca="1">'Kauno 36-118 II'!B13</f>
-        <v>230</v>
+        <v>221</v>
       </c>
       <c r="K26" s="10" t="str">
         <f ca="1">'Kauno 36-118 II'!S3</f>
@@ -4682,7 +4673,7 @@
       </c>
       <c r="J27" s="10">
         <f ca="1">'Vakaro 3A K1 III'!B13</f>
-        <v>345</v>
+        <v>336</v>
       </c>
       <c r="K27" s="10" t="str">
         <f ca="1">'Vakaro 3A K1 III'!S3</f>
@@ -4731,7 +4722,7 @@
       </c>
       <c r="H28" s="21">
         <f>'Užnerio butai XV'!B12</f>
-        <v>46597</v>
+        <v>46603</v>
       </c>
       <c r="I28" s="21" t="str">
         <f>'Užnerio butai XV'!R3</f>
@@ -4739,7 +4730,7 @@
       </c>
       <c r="J28" s="10">
         <f ca="1">'Užnerio butai XV'!B13</f>
-        <v>365</v>
+        <v>362</v>
       </c>
       <c r="K28" s="10" t="str">
         <f ca="1">'Užnerio butai XV'!S3</f>
@@ -4859,21 +4850,21 @@
       <c r="K1" s="9" t="s">
         <v>42</v>
       </c>
-      <c r="M1" s="30" t="s">
-        <v>0</v>
-      </c>
-      <c r="N1" s="32"/>
-      <c r="O1" s="30" t="s">
+      <c r="M1" s="28" t="s">
+        <v>0</v>
+      </c>
+      <c r="N1" s="30"/>
+      <c r="O1" s="28" t="s">
         <v>5</v>
       </c>
-      <c r="P1" s="32"/>
-      <c r="Q1" s="35" t="s">
+      <c r="P1" s="30"/>
+      <c r="Q1" s="33" t="s">
         <v>79</v>
       </c>
-      <c r="R1" s="35" t="s">
+      <c r="R1" s="33" t="s">
         <v>45</v>
       </c>
-      <c r="S1" s="35" t="s">
+      <c r="S1" s="33" t="s">
         <v>84</v>
       </c>
       <c r="Y1" s="17" t="s">
@@ -4930,9 +4921,9 @@
       <c r="P2" s="8" t="s">
         <v>78</v>
       </c>
-      <c r="Q2" s="36"/>
-      <c r="R2" s="36"/>
-      <c r="S2" s="36"/>
+      <c r="Q2" s="34"/>
+      <c r="R2" s="34"/>
+      <c r="S2" s="34"/>
       <c r="Y2" s="11">
         <f>B4</f>
         <v>46057</v>
@@ -5785,21 +5776,21 @@
       <c r="K1" s="9" t="s">
         <v>42</v>
       </c>
-      <c r="M1" s="30" t="s">
-        <v>0</v>
-      </c>
-      <c r="N1" s="32"/>
-      <c r="O1" s="30" t="s">
+      <c r="M1" s="28" t="s">
+        <v>0</v>
+      </c>
+      <c r="N1" s="30"/>
+      <c r="O1" s="28" t="s">
         <v>5</v>
       </c>
-      <c r="P1" s="32"/>
-      <c r="Q1" s="35" t="s">
+      <c r="P1" s="30"/>
+      <c r="Q1" s="33" t="s">
         <v>79</v>
       </c>
-      <c r="R1" s="35" t="s">
+      <c r="R1" s="33" t="s">
         <v>45</v>
       </c>
-      <c r="S1" s="35" t="s">
+      <c r="S1" s="33" t="s">
         <v>84</v>
       </c>
       <c r="Y1" s="17" t="s">
@@ -5856,9 +5847,9 @@
       <c r="P2" s="8" t="s">
         <v>78</v>
       </c>
-      <c r="Q2" s="36"/>
-      <c r="R2" s="36"/>
-      <c r="S2" s="36"/>
+      <c r="Q2" s="34"/>
+      <c r="R2" s="34"/>
+      <c r="S2" s="34"/>
       <c r="Y2" s="11">
         <f>B4</f>
         <v>46055</v>
@@ -6194,7 +6185,7 @@
       </c>
       <c r="B13" s="10">
         <f ca="1">IF(B11&lt;&gt;N3,(TODAY()-B12)*-1,"")</f>
-        <v>188</v>
+        <v>179</v>
       </c>
       <c r="D13" s="11"/>
       <c r="E13" s="15"/>
@@ -6710,21 +6701,21 @@
       <c r="K1" s="9" t="s">
         <v>42</v>
       </c>
-      <c r="M1" s="30" t="s">
-        <v>0</v>
-      </c>
-      <c r="N1" s="32"/>
-      <c r="O1" s="30" t="s">
+      <c r="M1" s="28" t="s">
+        <v>0</v>
+      </c>
+      <c r="N1" s="30"/>
+      <c r="O1" s="28" t="s">
         <v>5</v>
       </c>
-      <c r="P1" s="32"/>
-      <c r="Q1" s="35" t="s">
+      <c r="P1" s="30"/>
+      <c r="Q1" s="33" t="s">
         <v>79</v>
       </c>
-      <c r="R1" s="35" t="s">
+      <c r="R1" s="33" t="s">
         <v>45</v>
       </c>
-      <c r="S1" s="35" t="s">
+      <c r="S1" s="33" t="s">
         <v>84</v>
       </c>
       <c r="Y1" s="17" t="s">
@@ -6781,9 +6772,9 @@
       <c r="P2" s="8" t="s">
         <v>78</v>
       </c>
-      <c r="Q2" s="36"/>
-      <c r="R2" s="36"/>
-      <c r="S2" s="36"/>
+      <c r="Q2" s="34"/>
+      <c r="R2" s="34"/>
+      <c r="S2" s="34"/>
       <c r="Y2" s="11">
         <f>B4</f>
         <v>46043</v>
@@ -7658,21 +7649,21 @@
       <c r="K1" s="9" t="s">
         <v>42</v>
       </c>
-      <c r="M1" s="30" t="s">
-        <v>0</v>
-      </c>
-      <c r="N1" s="32"/>
-      <c r="O1" s="30" t="s">
+      <c r="M1" s="28" t="s">
+        <v>0</v>
+      </c>
+      <c r="N1" s="30"/>
+      <c r="O1" s="28" t="s">
         <v>5</v>
       </c>
-      <c r="P1" s="32"/>
-      <c r="Q1" s="35" t="s">
+      <c r="P1" s="30"/>
+      <c r="Q1" s="33" t="s">
         <v>79</v>
       </c>
-      <c r="R1" s="35" t="s">
+      <c r="R1" s="33" t="s">
         <v>45</v>
       </c>
-      <c r="S1" s="35" t="s">
+      <c r="S1" s="33" t="s">
         <v>84</v>
       </c>
       <c r="Y1" s="17" t="s">
@@ -7729,9 +7720,9 @@
       <c r="P2" s="8" t="s">
         <v>78</v>
       </c>
-      <c r="Q2" s="36"/>
-      <c r="R2" s="36"/>
-      <c r="S2" s="36"/>
+      <c r="Q2" s="34"/>
+      <c r="R2" s="34"/>
+      <c r="S2" s="34"/>
       <c r="Y2" s="11">
         <f>B4</f>
         <v>46013</v>
@@ -8075,7 +8066,7 @@
       </c>
       <c r="B13" s="10">
         <f ca="1">IF(B11&lt;&gt;N3,(TODAY()-B12)*-1,"")</f>
-        <v>146</v>
+        <v>137</v>
       </c>
       <c r="D13" s="11"/>
       <c r="E13" s="15"/>
@@ -8588,21 +8579,21 @@
       <c r="K1" s="9" t="s">
         <v>42</v>
       </c>
-      <c r="M1" s="30" t="s">
-        <v>0</v>
-      </c>
-      <c r="N1" s="32"/>
-      <c r="O1" s="30" t="s">
+      <c r="M1" s="28" t="s">
+        <v>0</v>
+      </c>
+      <c r="N1" s="30"/>
+      <c r="O1" s="28" t="s">
         <v>5</v>
       </c>
-      <c r="P1" s="32"/>
-      <c r="Q1" s="35" t="s">
+      <c r="P1" s="30"/>
+      <c r="Q1" s="33" t="s">
         <v>79</v>
       </c>
-      <c r="R1" s="35" t="s">
+      <c r="R1" s="33" t="s">
         <v>45</v>
       </c>
-      <c r="S1" s="35" t="s">
+      <c r="S1" s="33" t="s">
         <v>84</v>
       </c>
       <c r="Y1" s="17" t="s">
@@ -8659,9 +8650,9 @@
       <c r="P2" s="8" t="s">
         <v>78</v>
       </c>
-      <c r="Q2" s="36"/>
-      <c r="R2" s="36"/>
-      <c r="S2" s="36"/>
+      <c r="Q2" s="34"/>
+      <c r="R2" s="34"/>
+      <c r="S2" s="34"/>
       <c r="Y2" s="11">
         <f>B4</f>
         <v>46003</v>
@@ -9005,7 +8996,7 @@
       </c>
       <c r="B13" s="10">
         <f ca="1">IF(B11&lt;&gt;N3,(TODAY()-B12)*-1,"")</f>
-        <v>139</v>
+        <v>130</v>
       </c>
       <c r="D13" s="11"/>
       <c r="E13" s="15"/>
@@ -9518,21 +9509,21 @@
       <c r="K1" s="9" t="s">
         <v>42</v>
       </c>
-      <c r="M1" s="30" t="s">
-        <v>0</v>
-      </c>
-      <c r="N1" s="32"/>
-      <c r="O1" s="30" t="s">
+      <c r="M1" s="28" t="s">
+        <v>0</v>
+      </c>
+      <c r="N1" s="30"/>
+      <c r="O1" s="28" t="s">
         <v>5</v>
       </c>
-      <c r="P1" s="32"/>
-      <c r="Q1" s="35" t="s">
+      <c r="P1" s="30"/>
+      <c r="Q1" s="33" t="s">
         <v>79</v>
       </c>
-      <c r="R1" s="35" t="s">
+      <c r="R1" s="33" t="s">
         <v>45</v>
       </c>
-      <c r="S1" s="35" t="s">
+      <c r="S1" s="33" t="s">
         <v>84</v>
       </c>
       <c r="Y1" s="17" t="s">
@@ -9589,9 +9580,9 @@
       <c r="P2" s="8" t="s">
         <v>78</v>
       </c>
-      <c r="Q2" s="36"/>
-      <c r="R2" s="36"/>
-      <c r="S2" s="36"/>
+      <c r="Q2" s="34"/>
+      <c r="R2" s="34"/>
+      <c r="S2" s="34"/>
       <c r="Y2" s="11">
         <f>B4</f>
         <v>45967</v>
@@ -9935,7 +9926,7 @@
       </c>
       <c r="B13" s="10">
         <f ca="1">IF(B11&lt;&gt;N3,(TODAY()-B12)*-1,"")</f>
-        <v>100</v>
+        <v>91</v>
       </c>
       <c r="D13" s="11"/>
       <c r="E13" s="15"/>
@@ -10451,21 +10442,21 @@
       <c r="K1" s="9" t="s">
         <v>42</v>
       </c>
-      <c r="M1" s="30" t="s">
-        <v>0</v>
-      </c>
-      <c r="N1" s="32"/>
-      <c r="O1" s="30" t="s">
+      <c r="M1" s="28" t="s">
+        <v>0</v>
+      </c>
+      <c r="N1" s="30"/>
+      <c r="O1" s="28" t="s">
         <v>5</v>
       </c>
-      <c r="P1" s="32"/>
-      <c r="Q1" s="35" t="s">
+      <c r="P1" s="30"/>
+      <c r="Q1" s="33" t="s">
         <v>79</v>
       </c>
-      <c r="R1" s="35" t="s">
+      <c r="R1" s="33" t="s">
         <v>45</v>
       </c>
-      <c r="S1" s="35" t="s">
+      <c r="S1" s="33" t="s">
         <v>84</v>
       </c>
       <c r="Y1" s="17" t="s">
@@ -10522,9 +10513,9 @@
       <c r="P2" s="8" t="s">
         <v>78</v>
       </c>
-      <c r="Q2" s="36"/>
-      <c r="R2" s="36"/>
-      <c r="S2" s="36"/>
+      <c r="Q2" s="34"/>
+      <c r="R2" s="34"/>
+      <c r="S2" s="34"/>
       <c r="Y2" s="11">
         <f>B4</f>
         <v>45951</v>
@@ -11385,21 +11376,21 @@
       <c r="K1" s="9" t="s">
         <v>42</v>
       </c>
-      <c r="M1" s="30" t="s">
-        <v>0</v>
-      </c>
-      <c r="N1" s="32"/>
-      <c r="O1" s="30" t="s">
+      <c r="M1" s="28" t="s">
+        <v>0</v>
+      </c>
+      <c r="N1" s="30"/>
+      <c r="O1" s="28" t="s">
         <v>5</v>
       </c>
-      <c r="P1" s="32"/>
-      <c r="Q1" s="35" t="s">
+      <c r="P1" s="30"/>
+      <c r="Q1" s="33" t="s">
         <v>79</v>
       </c>
-      <c r="R1" s="35" t="s">
+      <c r="R1" s="33" t="s">
         <v>45</v>
       </c>
-      <c r="S1" s="35" t="s">
+      <c r="S1" s="33" t="s">
         <v>84</v>
       </c>
       <c r="Y1" s="17" t="s">
@@ -11456,9 +11447,9 @@
       <c r="P2" s="8" t="s">
         <v>78</v>
       </c>
-      <c r="Q2" s="36"/>
-      <c r="R2" s="36"/>
-      <c r="S2" s="36"/>
+      <c r="Q2" s="34"/>
+      <c r="R2" s="34"/>
+      <c r="S2" s="34"/>
       <c r="Y2" s="11">
         <f>B4</f>
         <v>45916</v>
@@ -11810,7 +11801,7 @@
       </c>
       <c r="B13" s="10">
         <f ca="1">IF(B11&lt;&gt;N3,(TODAY()-B12)*-1,"")</f>
-        <v>49</v>
+        <v>40</v>
       </c>
       <c r="D13" s="11"/>
       <c r="E13" s="15"/>
@@ -12326,21 +12317,21 @@
       <c r="K1" s="9" t="s">
         <v>42</v>
       </c>
-      <c r="M1" s="30" t="s">
-        <v>0</v>
-      </c>
-      <c r="N1" s="32"/>
-      <c r="O1" s="30" t="s">
+      <c r="M1" s="28" t="s">
+        <v>0</v>
+      </c>
+      <c r="N1" s="30"/>
+      <c r="O1" s="28" t="s">
         <v>5</v>
       </c>
-      <c r="P1" s="32"/>
-      <c r="Q1" s="35" t="s">
+      <c r="P1" s="30"/>
+      <c r="Q1" s="33" t="s">
         <v>79</v>
       </c>
-      <c r="R1" s="35" t="s">
+      <c r="R1" s="33" t="s">
         <v>45</v>
       </c>
-      <c r="S1" s="35" t="s">
+      <c r="S1" s="33" t="s">
         <v>84</v>
       </c>
       <c r="Y1" s="17" t="s">
@@ -12397,9 +12388,9 @@
       <c r="P2" s="8" t="s">
         <v>78</v>
       </c>
-      <c r="Q2" s="36"/>
-      <c r="R2" s="36"/>
-      <c r="S2" s="36"/>
+      <c r="Q2" s="34"/>
+      <c r="R2" s="34"/>
+      <c r="S2" s="34"/>
       <c r="Y2" s="11">
         <f>B4</f>
         <v>45917</v>
@@ -13260,21 +13251,21 @@
       <c r="K1" s="9" t="s">
         <v>42</v>
       </c>
-      <c r="M1" s="30" t="s">
-        <v>0</v>
-      </c>
-      <c r="N1" s="32"/>
-      <c r="O1" s="30" t="s">
+      <c r="M1" s="28" t="s">
+        <v>0</v>
+      </c>
+      <c r="N1" s="30"/>
+      <c r="O1" s="28" t="s">
         <v>5</v>
       </c>
-      <c r="P1" s="32"/>
-      <c r="Q1" s="35" t="s">
+      <c r="P1" s="30"/>
+      <c r="Q1" s="33" t="s">
         <v>79</v>
       </c>
-      <c r="R1" s="35" t="s">
+      <c r="R1" s="33" t="s">
         <v>45</v>
       </c>
-      <c r="S1" s="35" t="s">
+      <c r="S1" s="33" t="s">
         <v>84</v>
       </c>
       <c r="Y1" s="17" t="s">
@@ -13331,9 +13322,9 @@
       <c r="P2" s="8" t="s">
         <v>78</v>
       </c>
-      <c r="Q2" s="36"/>
-      <c r="R2" s="36"/>
-      <c r="S2" s="36"/>
+      <c r="Q2" s="34"/>
+      <c r="R2" s="34"/>
+      <c r="S2" s="34"/>
       <c r="Y2" s="11">
         <f>B4</f>
         <v>45908</v>
@@ -13685,7 +13676,7 @@
       </c>
       <c r="B13" s="10">
         <f ca="1">IF(B11&lt;&gt;N3,(TODAY()-B12)*-1,"")</f>
-        <v>42</v>
+        <v>33</v>
       </c>
       <c r="D13" s="11"/>
       <c r="E13" s="15"/>
@@ -14469,7 +14460,7 @@
     <row r="200" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A200" s="12">
         <f ca="1">TODAY()</f>
-        <v>46232</v>
+        <v>46241</v>
       </c>
       <c r="K200" s="25">
         <f>Overview!U3</f>
@@ -14535,21 +14526,21 @@
       <c r="K1" s="9" t="s">
         <v>42</v>
       </c>
-      <c r="M1" s="30" t="s">
-        <v>0</v>
-      </c>
-      <c r="N1" s="32"/>
-      <c r="O1" s="30" t="s">
+      <c r="M1" s="28" t="s">
+        <v>0</v>
+      </c>
+      <c r="N1" s="30"/>
+      <c r="O1" s="28" t="s">
         <v>5</v>
       </c>
-      <c r="P1" s="32"/>
-      <c r="Q1" s="35" t="s">
+      <c r="P1" s="30"/>
+      <c r="Q1" s="33" t="s">
         <v>79</v>
       </c>
-      <c r="R1" s="35" t="s">
+      <c r="R1" s="33" t="s">
         <v>45</v>
       </c>
-      <c r="S1" s="35" t="s">
+      <c r="S1" s="33" t="s">
         <v>84</v>
       </c>
       <c r="Y1" s="17" t="s">
@@ -14606,9 +14597,9 @@
       <c r="P2" s="8" t="s">
         <v>78</v>
       </c>
-      <c r="Q2" s="36"/>
-      <c r="R2" s="36"/>
-      <c r="S2" s="36"/>
+      <c r="Q2" s="34"/>
+      <c r="R2" s="34"/>
+      <c r="S2" s="34"/>
       <c r="Y2" s="11">
         <f>B3</f>
         <v>45791</v>
@@ -15458,21 +15449,21 @@
       <c r="K1" s="9" t="s">
         <v>42</v>
       </c>
-      <c r="M1" s="30" t="s">
-        <v>0</v>
-      </c>
-      <c r="N1" s="32"/>
-      <c r="O1" s="30" t="s">
+      <c r="M1" s="28" t="s">
+        <v>0</v>
+      </c>
+      <c r="N1" s="30"/>
+      <c r="O1" s="28" t="s">
         <v>5</v>
       </c>
-      <c r="P1" s="32"/>
-      <c r="Q1" s="35" t="s">
+      <c r="P1" s="30"/>
+      <c r="Q1" s="33" t="s">
         <v>79</v>
       </c>
-      <c r="R1" s="35" t="s">
+      <c r="R1" s="33" t="s">
         <v>45</v>
       </c>
-      <c r="S1" s="35" t="s">
+      <c r="S1" s="33" t="s">
         <v>84</v>
       </c>
       <c r="Y1" s="17" t="s">
@@ -15529,9 +15520,9 @@
       <c r="P2" s="8" t="s">
         <v>78</v>
       </c>
-      <c r="Q2" s="36"/>
-      <c r="R2" s="36"/>
-      <c r="S2" s="36"/>
+      <c r="Q2" s="34"/>
+      <c r="R2" s="34"/>
+      <c r="S2" s="34"/>
       <c r="Y2" s="11">
         <f>B3</f>
         <v>45770</v>
@@ -16409,21 +16400,21 @@
       <c r="K1" s="9" t="s">
         <v>42</v>
       </c>
-      <c r="M1" s="30" t="s">
-        <v>0</v>
-      </c>
-      <c r="N1" s="32"/>
-      <c r="O1" s="30" t="s">
+      <c r="M1" s="28" t="s">
+        <v>0</v>
+      </c>
+      <c r="N1" s="30"/>
+      <c r="O1" s="28" t="s">
         <v>5</v>
       </c>
-      <c r="P1" s="32"/>
-      <c r="Q1" s="35" t="s">
+      <c r="P1" s="30"/>
+      <c r="Q1" s="33" t="s">
         <v>79</v>
       </c>
-      <c r="R1" s="35" t="s">
+      <c r="R1" s="33" t="s">
         <v>45</v>
       </c>
-      <c r="S1" s="35" t="s">
+      <c r="S1" s="33" t="s">
         <v>84</v>
       </c>
       <c r="Y1" s="17" t="s">
@@ -16480,9 +16471,9 @@
       <c r="P2" s="8" t="s">
         <v>78</v>
       </c>
-      <c r="Q2" s="36"/>
-      <c r="R2" s="36"/>
-      <c r="S2" s="36"/>
+      <c r="Q2" s="34"/>
+      <c r="R2" s="34"/>
+      <c r="S2" s="34"/>
       <c r="Y2" s="11">
         <f>B3</f>
         <v>45764</v>
@@ -17374,21 +17365,21 @@
       <c r="K1" s="9" t="s">
         <v>42</v>
       </c>
-      <c r="M1" s="30" t="s">
-        <v>0</v>
-      </c>
-      <c r="N1" s="32"/>
-      <c r="O1" s="30" t="s">
+      <c r="M1" s="28" t="s">
+        <v>0</v>
+      </c>
+      <c r="N1" s="30"/>
+      <c r="O1" s="28" t="s">
         <v>5</v>
       </c>
-      <c r="P1" s="32"/>
-      <c r="Q1" s="35" t="s">
+      <c r="P1" s="30"/>
+      <c r="Q1" s="33" t="s">
         <v>79</v>
       </c>
-      <c r="R1" s="35" t="s">
+      <c r="R1" s="33" t="s">
         <v>45</v>
       </c>
-      <c r="S1" s="35" t="s">
+      <c r="S1" s="33" t="s">
         <v>84</v>
       </c>
       <c r="Y1" s="17" t="s">
@@ -17445,9 +17436,9 @@
       <c r="P2" s="8" t="s">
         <v>78</v>
       </c>
-      <c r="Q2" s="36"/>
-      <c r="R2" s="36"/>
-      <c r="S2" s="36"/>
+      <c r="Q2" s="34"/>
+      <c r="R2" s="34"/>
+      <c r="S2" s="34"/>
       <c r="Y2" s="11">
         <f>B3</f>
         <v>45757</v>
@@ -18296,21 +18287,21 @@
       <c r="K1" s="9" t="s">
         <v>42</v>
       </c>
-      <c r="M1" s="30" t="s">
-        <v>0</v>
-      </c>
-      <c r="N1" s="32"/>
-      <c r="O1" s="30" t="s">
+      <c r="M1" s="28" t="s">
+        <v>0</v>
+      </c>
+      <c r="N1" s="30"/>
+      <c r="O1" s="28" t="s">
         <v>5</v>
       </c>
-      <c r="P1" s="32"/>
-      <c r="Q1" s="35" t="s">
+      <c r="P1" s="30"/>
+      <c r="Q1" s="33" t="s">
         <v>79</v>
       </c>
-      <c r="R1" s="35" t="s">
+      <c r="R1" s="33" t="s">
         <v>45</v>
       </c>
-      <c r="S1" s="35" t="s">
+      <c r="S1" s="33" t="s">
         <v>84</v>
       </c>
       <c r="Y1" s="17" t="s">
@@ -18367,9 +18358,9 @@
       <c r="P2" s="8" t="s">
         <v>78</v>
       </c>
-      <c r="Q2" s="36"/>
-      <c r="R2" s="36"/>
-      <c r="S2" s="36"/>
+      <c r="Q2" s="34"/>
+      <c r="R2" s="34"/>
+      <c r="S2" s="34"/>
       <c r="Y2" s="11">
         <f>B3</f>
         <v>45743</v>
@@ -19260,21 +19251,21 @@
       <c r="K1" s="9" t="s">
         <v>42</v>
       </c>
-      <c r="M1" s="30" t="s">
-        <v>0</v>
-      </c>
-      <c r="N1" s="32"/>
-      <c r="O1" s="30" t="s">
+      <c r="M1" s="28" t="s">
+        <v>0</v>
+      </c>
+      <c r="N1" s="30"/>
+      <c r="O1" s="28" t="s">
         <v>5</v>
       </c>
-      <c r="P1" s="32"/>
-      <c r="Q1" s="35" t="s">
+      <c r="P1" s="30"/>
+      <c r="Q1" s="33" t="s">
         <v>79</v>
       </c>
-      <c r="R1" s="35" t="s">
+      <c r="R1" s="33" t="s">
         <v>45</v>
       </c>
-      <c r="S1" s="35" t="s">
+      <c r="S1" s="33" t="s">
         <v>84</v>
       </c>
       <c r="Y1" s="17" t="s">
@@ -19331,9 +19322,9 @@
       <c r="P2" s="8" t="s">
         <v>78</v>
       </c>
-      <c r="Q2" s="36"/>
-      <c r="R2" s="36"/>
-      <c r="S2" s="36"/>
+      <c r="Q2" s="34"/>
+      <c r="R2" s="34"/>
+      <c r="S2" s="34"/>
       <c r="Y2" s="11">
         <f>B3</f>
         <v>45729</v>
@@ -20412,21 +20403,21 @@
       <c r="K1" s="9" t="s">
         <v>42</v>
       </c>
-      <c r="M1" s="30" t="s">
-        <v>0</v>
-      </c>
-      <c r="N1" s="32"/>
-      <c r="O1" s="30" t="s">
+      <c r="M1" s="28" t="s">
+        <v>0</v>
+      </c>
+      <c r="N1" s="30"/>
+      <c r="O1" s="28" t="s">
         <v>5</v>
       </c>
-      <c r="P1" s="32"/>
-      <c r="Q1" s="35" t="s">
+      <c r="P1" s="30"/>
+      <c r="Q1" s="33" t="s">
         <v>79</v>
       </c>
-      <c r="R1" s="35" t="s">
+      <c r="R1" s="33" t="s">
         <v>45</v>
       </c>
-      <c r="S1" s="35" t="s">
+      <c r="S1" s="33" t="s">
         <v>84</v>
       </c>
       <c r="Y1" s="17" t="s">
@@ -20483,9 +20474,9 @@
       <c r="P2" s="8" t="s">
         <v>78</v>
       </c>
-      <c r="Q2" s="36"/>
-      <c r="R2" s="36"/>
-      <c r="S2" s="36"/>
+      <c r="Q2" s="34"/>
+      <c r="R2" s="34"/>
+      <c r="S2" s="34"/>
       <c r="Y2" s="11">
         <f>B3</f>
         <v>45725</v>
@@ -21565,21 +21556,21 @@
       <c r="K1" s="9" t="s">
         <v>42</v>
       </c>
-      <c r="M1" s="30" t="s">
-        <v>0</v>
-      </c>
-      <c r="N1" s="32"/>
-      <c r="O1" s="30" t="s">
+      <c r="M1" s="28" t="s">
+        <v>0</v>
+      </c>
+      <c r="N1" s="30"/>
+      <c r="O1" s="28" t="s">
         <v>5</v>
       </c>
-      <c r="P1" s="32"/>
-      <c r="Q1" s="35" t="s">
+      <c r="P1" s="30"/>
+      <c r="Q1" s="33" t="s">
         <v>79</v>
       </c>
-      <c r="R1" s="35" t="s">
+      <c r="R1" s="33" t="s">
         <v>45</v>
       </c>
-      <c r="S1" s="35" t="s">
+      <c r="S1" s="33" t="s">
         <v>84</v>
       </c>
       <c r="Y1" s="17" t="s">
@@ -21636,9 +21627,9 @@
       <c r="P2" s="8" t="s">
         <v>78</v>
       </c>
-      <c r="Q2" s="36"/>
-      <c r="R2" s="36"/>
-      <c r="S2" s="36"/>
+      <c r="Q2" s="34"/>
+      <c r="R2" s="34"/>
+      <c r="S2" s="34"/>
       <c r="Y2" s="11">
         <f>B3</f>
         <v>45721</v>
@@ -22734,21 +22725,21 @@
       <c r="K1" s="9" t="s">
         <v>42</v>
       </c>
-      <c r="M1" s="30" t="s">
-        <v>0</v>
-      </c>
-      <c r="N1" s="32"/>
-      <c r="O1" s="30" t="s">
+      <c r="M1" s="28" t="s">
+        <v>0</v>
+      </c>
+      <c r="N1" s="30"/>
+      <c r="O1" s="28" t="s">
         <v>5</v>
       </c>
-      <c r="P1" s="32"/>
-      <c r="Q1" s="35" t="s">
+      <c r="P1" s="30"/>
+      <c r="Q1" s="33" t="s">
         <v>79</v>
       </c>
-      <c r="R1" s="35" t="s">
+      <c r="R1" s="33" t="s">
         <v>45</v>
       </c>
-      <c r="S1" s="35" t="s">
+      <c r="S1" s="33" t="s">
         <v>84</v>
       </c>
       <c r="Y1" s="17" t="s">
@@ -22805,9 +22796,9 @@
       <c r="P2" s="8" t="s">
         <v>78</v>
       </c>
-      <c r="Q2" s="36"/>
-      <c r="R2" s="36"/>
-      <c r="S2" s="36"/>
+      <c r="Q2" s="34"/>
+      <c r="R2" s="34"/>
+      <c r="S2" s="34"/>
       <c r="Y2" s="11">
         <f>B3</f>
         <v>45719</v>
@@ -23876,22 +23867,22 @@
       <c r="B1" s="2" t="s">
         <v>100</v>
       </c>
-      <c r="D1" s="28" t="s">
+      <c r="D1" s="8" t="s">
         <v>9</v>
       </c>
-      <c r="E1" s="28" t="s">
-        <v>0</v>
-      </c>
-      <c r="F1" s="28" t="s">
+      <c r="E1" s="8" t="s">
+        <v>0</v>
+      </c>
+      <c r="F1" s="8" t="s">
         <v>5</v>
       </c>
-      <c r="G1" s="28" t="s">
-        <v>0</v>
-      </c>
-      <c r="H1" s="28" t="s">
+      <c r="G1" s="8" t="s">
+        <v>0</v>
+      </c>
+      <c r="H1" s="8" t="s">
         <v>5</v>
       </c>
-      <c r="I1" s="28" t="s">
+      <c r="I1" s="8" t="s">
         <v>62</v>
       </c>
       <c r="J1" s="9" t="s">
@@ -23900,30 +23891,30 @@
       <c r="K1" s="9" t="s">
         <v>42</v>
       </c>
-      <c r="M1" s="30" t="s">
-        <v>0</v>
-      </c>
-      <c r="N1" s="32"/>
-      <c r="O1" s="30" t="s">
+      <c r="M1" s="28" t="s">
+        <v>0</v>
+      </c>
+      <c r="N1" s="30"/>
+      <c r="O1" s="28" t="s">
         <v>5</v>
       </c>
-      <c r="P1" s="32"/>
-      <c r="Q1" s="35" t="s">
+      <c r="P1" s="30"/>
+      <c r="Q1" s="33" t="s">
         <v>79</v>
       </c>
-      <c r="R1" s="35" t="s">
+      <c r="R1" s="33" t="s">
         <v>45</v>
       </c>
-      <c r="S1" s="35" t="s">
+      <c r="S1" s="33" t="s">
         <v>84</v>
       </c>
       <c r="Y1" s="17" t="s">
         <v>9</v>
       </c>
-      <c r="Z1" s="28" t="s">
+      <c r="Z1" s="8" t="s">
         <v>75</v>
       </c>
-      <c r="AA1" s="28" t="s">
+      <c r="AA1" s="8" t="s">
         <v>84</v>
       </c>
     </row>
@@ -23934,9 +23925,15 @@
       <c r="B2" s="2" t="s">
         <v>99</v>
       </c>
-      <c r="D2" s="11"/>
-      <c r="E2" s="4"/>
-      <c r="F2" s="4"/>
+      <c r="D2" s="11">
+        <v>46329</v>
+      </c>
+      <c r="E2" s="4">
+        <v>0</v>
+      </c>
+      <c r="F2" s="4">
+        <v>2.74</v>
+      </c>
       <c r="G2" s="4"/>
       <c r="H2" s="4"/>
       <c r="I2" s="4"/>
@@ -23951,18 +23948,18 @@
       <c r="N2" s="16" t="s">
         <v>45</v>
       </c>
-      <c r="O2" s="28" t="s">
+      <c r="O2" s="8" t="s">
         <v>77</v>
       </c>
-      <c r="P2" s="28" t="s">
+      <c r="P2" s="8" t="s">
         <v>78</v>
       </c>
-      <c r="Q2" s="36"/>
-      <c r="R2" s="36"/>
-      <c r="S2" s="36"/>
+      <c r="Q2" s="34"/>
+      <c r="R2" s="34"/>
+      <c r="S2" s="34"/>
       <c r="Y2" s="11">
         <f>B4</f>
-        <v>0</v>
+        <v>46238</v>
       </c>
       <c r="Z2" s="4">
         <f>B11*-1</f>
@@ -23980,9 +23977,15 @@
       <c r="B3" s="11">
         <v>46232</v>
       </c>
-      <c r="D3" s="11"/>
-      <c r="E3" s="4"/>
-      <c r="F3" s="4"/>
+      <c r="D3" s="11">
+        <v>46419</v>
+      </c>
+      <c r="E3" s="4">
+        <v>0</v>
+      </c>
+      <c r="F3" s="4">
+        <v>2.57</v>
+      </c>
       <c r="G3" s="4"/>
       <c r="H3" s="4"/>
       <c r="I3" s="4"/>
@@ -24001,7 +24004,7 @@
       </c>
       <c r="O3" s="4">
         <f>F42</f>
-        <v>0</v>
+        <v>10.65</v>
       </c>
       <c r="P3" s="4">
         <f>H42+I42</f>
@@ -24032,10 +24035,18 @@
       <c r="A4" s="7" t="s">
         <v>11</v>
       </c>
-      <c r="B4" s="11"/>
-      <c r="D4" s="11"/>
-      <c r="E4" s="4"/>
-      <c r="F4" s="4"/>
+      <c r="B4" s="11">
+        <v>46238</v>
+      </c>
+      <c r="D4" s="11">
+        <v>46507</v>
+      </c>
+      <c r="E4" s="4">
+        <v>0</v>
+      </c>
+      <c r="F4" s="4">
+        <v>2.6</v>
+      </c>
       <c r="G4" s="4"/>
       <c r="H4" s="4"/>
       <c r="I4" s="4"/>
@@ -24060,9 +24071,15 @@
       <c r="B5" s="2" t="s">
         <v>15</v>
       </c>
-      <c r="D5" s="11"/>
-      <c r="E5" s="4"/>
-      <c r="F5" s="4"/>
+      <c r="D5" s="11">
+        <v>46603</v>
+      </c>
+      <c r="E5" s="4">
+        <v>110.51</v>
+      </c>
+      <c r="F5" s="4">
+        <v>2.74</v>
+      </c>
       <c r="G5" s="4"/>
       <c r="H5" s="4"/>
       <c r="I5" s="4"/>
@@ -24115,7 +24132,7 @@
         <v>0.75</v>
       </c>
       <c r="D7" s="11"/>
-      <c r="E7" s="2"/>
+      <c r="E7" s="4"/>
       <c r="F7" s="4"/>
       <c r="G7" s="2"/>
       <c r="H7" s="4"/>
@@ -24142,7 +24159,7 @@
         <v>12</v>
       </c>
       <c r="D8" s="11"/>
-      <c r="E8" s="15"/>
+      <c r="E8" s="4"/>
       <c r="F8" s="15"/>
       <c r="G8" s="15"/>
       <c r="H8" s="15"/>
@@ -24169,7 +24186,7 @@
         <v>8</v>
       </c>
       <c r="D9" s="11"/>
-      <c r="E9" s="15"/>
+      <c r="E9" s="4"/>
       <c r="F9" s="15"/>
       <c r="G9" s="15"/>
       <c r="H9" s="15"/>
@@ -24196,7 +24213,7 @@
         <v>9.5000000000000001E-2</v>
       </c>
       <c r="D10" s="11"/>
-      <c r="E10" s="15"/>
+      <c r="E10" s="4"/>
       <c r="F10" s="15"/>
       <c r="G10" s="15"/>
       <c r="H10" s="15"/>
@@ -24223,7 +24240,7 @@
         <v>110.51</v>
       </c>
       <c r="D11" s="11"/>
-      <c r="E11" s="15"/>
+      <c r="E11" s="4"/>
       <c r="F11" s="15"/>
       <c r="G11" s="15"/>
       <c r="H11" s="15"/>
@@ -24246,11 +24263,11 @@
       <c r="A12" s="7" t="s">
         <v>85</v>
       </c>
-      <c r="B12" s="29">
-        <v>46597</v>
+      <c r="B12" s="35">
+        <v>46603</v>
       </c>
       <c r="D12" s="11"/>
-      <c r="E12" s="15"/>
+      <c r="E12" s="4"/>
       <c r="F12" s="15"/>
       <c r="G12" s="15"/>
       <c r="H12" s="15"/>
@@ -24275,10 +24292,10 @@
       </c>
       <c r="B13" s="10">
         <f ca="1">IF(B11&lt;&gt;N3,(TODAY()-B12)*-1,"")</f>
-        <v>365</v>
+        <v>362</v>
       </c>
       <c r="D13" s="11"/>
-      <c r="E13" s="15"/>
+      <c r="E13" s="4"/>
       <c r="F13" s="15"/>
       <c r="G13" s="15"/>
       <c r="H13" s="15"/>
@@ -24302,7 +24319,7 @@
         <v>45</v>
       </c>
       <c r="B14" s="11"/>
-      <c r="D14" s="28"/>
+      <c r="D14" s="8"/>
       <c r="E14" s="4"/>
       <c r="F14" s="4"/>
       <c r="G14" s="4"/>
@@ -24330,7 +24347,7 @@
         <f>IF(M3=N3,B14-B12,"")</f>
         <v/>
       </c>
-      <c r="D15" s="28"/>
+      <c r="D15" s="8"/>
       <c r="E15" s="4"/>
       <c r="F15" s="4"/>
       <c r="G15" s="4"/>
@@ -24343,7 +24360,7 @@
       </c>
     </row>
     <row r="16" spans="1:27" x14ac:dyDescent="0.25">
-      <c r="D16" s="28"/>
+      <c r="D16" s="8"/>
       <c r="E16" s="4"/>
       <c r="F16" s="4"/>
       <c r="G16" s="4"/>
@@ -24356,7 +24373,7 @@
       </c>
     </row>
     <row r="17" spans="4:11" x14ac:dyDescent="0.25">
-      <c r="D17" s="28"/>
+      <c r="D17" s="8"/>
       <c r="E17" s="4"/>
       <c r="F17" s="4"/>
       <c r="G17" s="4"/>
@@ -24369,7 +24386,7 @@
       </c>
     </row>
     <row r="18" spans="4:11" x14ac:dyDescent="0.25">
-      <c r="D18" s="28"/>
+      <c r="D18" s="8"/>
       <c r="E18" s="4"/>
       <c r="F18" s="4"/>
       <c r="G18" s="4"/>
@@ -24382,7 +24399,7 @@
       </c>
     </row>
     <row r="19" spans="4:11" x14ac:dyDescent="0.25">
-      <c r="D19" s="28"/>
+      <c r="D19" s="8"/>
       <c r="E19" s="4"/>
       <c r="F19" s="4"/>
       <c r="G19" s="4"/>
@@ -24395,7 +24412,7 @@
       </c>
     </row>
     <row r="20" spans="4:11" x14ac:dyDescent="0.25">
-      <c r="D20" s="28"/>
+      <c r="D20" s="8"/>
       <c r="E20" s="4"/>
       <c r="F20" s="4"/>
       <c r="G20" s="4"/>
@@ -24408,7 +24425,7 @@
       </c>
     </row>
     <row r="21" spans="4:11" x14ac:dyDescent="0.25">
-      <c r="D21" s="28"/>
+      <c r="D21" s="8"/>
       <c r="E21" s="4"/>
       <c r="F21" s="4"/>
       <c r="G21" s="4"/>
@@ -24421,7 +24438,7 @@
       </c>
     </row>
     <row r="22" spans="4:11" x14ac:dyDescent="0.25">
-      <c r="D22" s="28"/>
+      <c r="D22" s="8"/>
       <c r="E22" s="4"/>
       <c r="F22" s="4"/>
       <c r="G22" s="4"/>
@@ -24434,7 +24451,7 @@
       </c>
     </row>
     <row r="23" spans="4:11" x14ac:dyDescent="0.25">
-      <c r="D23" s="28"/>
+      <c r="D23" s="8"/>
       <c r="E23" s="4"/>
       <c r="F23" s="4"/>
       <c r="G23" s="4"/>
@@ -24447,7 +24464,7 @@
       </c>
     </row>
     <row r="24" spans="4:11" x14ac:dyDescent="0.25">
-      <c r="D24" s="28"/>
+      <c r="D24" s="8"/>
       <c r="E24" s="4"/>
       <c r="F24" s="4"/>
       <c r="G24" s="4"/>
@@ -24460,7 +24477,7 @@
       </c>
     </row>
     <row r="25" spans="4:11" x14ac:dyDescent="0.25">
-      <c r="D25" s="28"/>
+      <c r="D25" s="8"/>
       <c r="E25" s="4"/>
       <c r="F25" s="4"/>
       <c r="G25" s="4"/>
@@ -24473,7 +24490,7 @@
       </c>
     </row>
     <row r="26" spans="4:11" x14ac:dyDescent="0.25">
-      <c r="D26" s="28"/>
+      <c r="D26" s="8"/>
       <c r="E26" s="4"/>
       <c r="F26" s="4"/>
       <c r="G26" s="4"/>
@@ -24486,7 +24503,7 @@
       </c>
     </row>
     <row r="27" spans="4:11" x14ac:dyDescent="0.25">
-      <c r="D27" s="28"/>
+      <c r="D27" s="8"/>
       <c r="E27" s="4"/>
       <c r="F27" s="4"/>
       <c r="G27" s="4"/>
@@ -24499,7 +24516,7 @@
       </c>
     </row>
     <row r="28" spans="4:11" x14ac:dyDescent="0.25">
-      <c r="D28" s="28"/>
+      <c r="D28" s="8"/>
       <c r="E28" s="4"/>
       <c r="F28" s="4"/>
       <c r="G28" s="4"/>
@@ -24512,7 +24529,7 @@
       </c>
     </row>
     <row r="29" spans="4:11" x14ac:dyDescent="0.25">
-      <c r="D29" s="28"/>
+      <c r="D29" s="8"/>
       <c r="E29" s="4"/>
       <c r="F29" s="4"/>
       <c r="G29" s="4"/>
@@ -24525,7 +24542,7 @@
       </c>
     </row>
     <row r="30" spans="4:11" x14ac:dyDescent="0.25">
-      <c r="D30" s="28"/>
+      <c r="D30" s="8"/>
       <c r="E30" s="4"/>
       <c r="F30" s="4"/>
       <c r="G30" s="4"/>
@@ -24538,7 +24555,7 @@
       </c>
     </row>
     <row r="31" spans="4:11" x14ac:dyDescent="0.25">
-      <c r="D31" s="28"/>
+      <c r="D31" s="8"/>
       <c r="E31" s="4"/>
       <c r="F31" s="4"/>
       <c r="G31" s="4"/>
@@ -24551,7 +24568,7 @@
       </c>
     </row>
     <row r="32" spans="4:11" x14ac:dyDescent="0.25">
-      <c r="D32" s="28"/>
+      <c r="D32" s="8"/>
       <c r="E32" s="4"/>
       <c r="F32" s="4"/>
       <c r="G32" s="4"/>
@@ -24564,7 +24581,7 @@
       </c>
     </row>
     <row r="33" spans="4:11" x14ac:dyDescent="0.25">
-      <c r="D33" s="28"/>
+      <c r="D33" s="8"/>
       <c r="E33" s="4"/>
       <c r="F33" s="4"/>
       <c r="G33" s="4"/>
@@ -24577,7 +24594,7 @@
       </c>
     </row>
     <row r="34" spans="4:11" x14ac:dyDescent="0.25">
-      <c r="D34" s="28"/>
+      <c r="D34" s="8"/>
       <c r="E34" s="4"/>
       <c r="F34" s="4"/>
       <c r="G34" s="4"/>
@@ -24590,7 +24607,7 @@
       </c>
     </row>
     <row r="35" spans="4:11" x14ac:dyDescent="0.25">
-      <c r="D35" s="28"/>
+      <c r="D35" s="8"/>
       <c r="E35" s="4"/>
       <c r="F35" s="4"/>
       <c r="G35" s="4"/>
@@ -24603,7 +24620,7 @@
       </c>
     </row>
     <row r="36" spans="4:11" x14ac:dyDescent="0.25">
-      <c r="D36" s="28"/>
+      <c r="D36" s="8"/>
       <c r="E36" s="4"/>
       <c r="F36" s="4"/>
       <c r="G36" s="4"/>
@@ -24616,7 +24633,7 @@
       </c>
     </row>
     <row r="37" spans="4:11" x14ac:dyDescent="0.25">
-      <c r="D37" s="28"/>
+      <c r="D37" s="8"/>
       <c r="E37" s="4"/>
       <c r="F37" s="4"/>
       <c r="G37" s="4"/>
@@ -24629,7 +24646,7 @@
       </c>
     </row>
     <row r="38" spans="4:11" x14ac:dyDescent="0.25">
-      <c r="D38" s="28"/>
+      <c r="D38" s="8"/>
       <c r="E38" s="4"/>
       <c r="F38" s="4"/>
       <c r="G38" s="4"/>
@@ -24642,7 +24659,7 @@
       </c>
     </row>
     <row r="39" spans="4:11" x14ac:dyDescent="0.25">
-      <c r="D39" s="28"/>
+      <c r="D39" s="8"/>
       <c r="E39" s="4"/>
       <c r="F39" s="4"/>
       <c r="G39" s="4"/>
@@ -24655,7 +24672,7 @@
       </c>
     </row>
     <row r="40" spans="4:11" x14ac:dyDescent="0.25">
-      <c r="D40" s="28"/>
+      <c r="D40" s="8"/>
       <c r="E40" s="4"/>
       <c r="F40" s="4"/>
       <c r="G40" s="4"/>
@@ -24668,7 +24685,7 @@
       </c>
     </row>
     <row r="41" spans="4:11" x14ac:dyDescent="0.25">
-      <c r="D41" s="28"/>
+      <c r="D41" s="8"/>
       <c r="E41" s="4"/>
       <c r="F41" s="4"/>
       <c r="G41" s="4"/>
@@ -24681,16 +24698,16 @@
       </c>
     </row>
     <row r="42" spans="4:11" x14ac:dyDescent="0.25">
-      <c r="D42" s="28" t="s">
+      <c r="D42" s="8" t="s">
         <v>10</v>
       </c>
       <c r="E42" s="4">
         <f>SUM(E2:E41)</f>
-        <v>0</v>
+        <v>110.51</v>
       </c>
       <c r="F42" s="4">
         <f t="shared" ref="F42:I42" si="3">SUM(F2:F41)</f>
-        <v>0</v>
+        <v>10.65</v>
       </c>
       <c r="G42" s="4">
         <f t="shared" si="3"/>
@@ -24788,21 +24805,21 @@
       <c r="K1" s="9" t="s">
         <v>42</v>
       </c>
-      <c r="M1" s="30" t="s">
-        <v>0</v>
-      </c>
-      <c r="N1" s="32"/>
-      <c r="O1" s="30" t="s">
+      <c r="M1" s="28" t="s">
+        <v>0</v>
+      </c>
+      <c r="N1" s="30"/>
+      <c r="O1" s="28" t="s">
         <v>5</v>
       </c>
-      <c r="P1" s="32"/>
-      <c r="Q1" s="35" t="s">
+      <c r="P1" s="30"/>
+      <c r="Q1" s="33" t="s">
         <v>79</v>
       </c>
-      <c r="R1" s="35" t="s">
+      <c r="R1" s="33" t="s">
         <v>45</v>
       </c>
-      <c r="S1" s="35" t="s">
+      <c r="S1" s="33" t="s">
         <v>84</v>
       </c>
       <c r="Y1" s="17" t="s">
@@ -24851,12 +24868,12 @@
       <c r="P2" s="8" t="s">
         <v>78</v>
       </c>
-      <c r="Q2" s="36"/>
-      <c r="R2" s="36"/>
-      <c r="S2" s="36"/>
+      <c r="Q2" s="34"/>
+      <c r="R2" s="34"/>
+      <c r="S2" s="34"/>
       <c r="Y2" s="11">
         <f>B4</f>
-        <v>0</v>
+        <v>46212</v>
       </c>
       <c r="Z2" s="4">
         <f>B11*-1</f>
@@ -24932,7 +24949,9 @@
       <c r="A4" s="7" t="s">
         <v>11</v>
       </c>
-      <c r="B4" s="11"/>
+      <c r="B4" s="11">
+        <v>46212</v>
+      </c>
       <c r="D4" s="11">
         <v>46507</v>
       </c>
@@ -25187,7 +25206,7 @@
       </c>
       <c r="B13" s="10">
         <f ca="1">IF(B11&lt;&gt;N3,(TODAY()-B12)*-1,"")</f>
-        <v>345</v>
+        <v>336</v>
       </c>
       <c r="D13" s="11"/>
       <c r="E13" s="15"/>
@@ -25700,21 +25719,21 @@
       <c r="K1" s="9" t="s">
         <v>42</v>
       </c>
-      <c r="M1" s="30" t="s">
-        <v>0</v>
-      </c>
-      <c r="N1" s="32"/>
-      <c r="O1" s="30" t="s">
+      <c r="M1" s="28" t="s">
+        <v>0</v>
+      </c>
+      <c r="N1" s="30"/>
+      <c r="O1" s="28" t="s">
         <v>5</v>
       </c>
-      <c r="P1" s="32"/>
-      <c r="Q1" s="35" t="s">
+      <c r="P1" s="30"/>
+      <c r="Q1" s="33" t="s">
         <v>79</v>
       </c>
-      <c r="R1" s="35" t="s">
+      <c r="R1" s="33" t="s">
         <v>45</v>
       </c>
-      <c r="S1" s="35" t="s">
+      <c r="S1" s="33" t="s">
         <v>84</v>
       </c>
       <c r="Y1" s="17" t="s">
@@ -25771,9 +25790,9 @@
       <c r="P2" s="8" t="s">
         <v>78</v>
       </c>
-      <c r="Q2" s="36"/>
-      <c r="R2" s="36"/>
-      <c r="S2" s="36"/>
+      <c r="Q2" s="34"/>
+      <c r="R2" s="34"/>
+      <c r="S2" s="34"/>
       <c r="Y2" s="11">
         <f>B4</f>
         <v>46097</v>
@@ -26109,7 +26128,7 @@
       </c>
       <c r="B13" s="10">
         <f ca="1">IF(B11&lt;&gt;N3,(TODAY()-B12)*-1,"")</f>
-        <v>230</v>
+        <v>221</v>
       </c>
       <c r="D13" s="11"/>
       <c r="E13" s="15"/>
@@ -26622,21 +26641,21 @@
       <c r="K1" s="9" t="s">
         <v>42</v>
       </c>
-      <c r="M1" s="30" t="s">
-        <v>0</v>
-      </c>
-      <c r="N1" s="32"/>
-      <c r="O1" s="30" t="s">
+      <c r="M1" s="28" t="s">
+        <v>0</v>
+      </c>
+      <c r="N1" s="30"/>
+      <c r="O1" s="28" t="s">
         <v>5</v>
       </c>
-      <c r="P1" s="32"/>
-      <c r="Q1" s="35" t="s">
+      <c r="P1" s="30"/>
+      <c r="Q1" s="33" t="s">
         <v>79</v>
       </c>
-      <c r="R1" s="35" t="s">
+      <c r="R1" s="33" t="s">
         <v>45</v>
       </c>
-      <c r="S1" s="35" t="s">
+      <c r="S1" s="33" t="s">
         <v>84</v>
       </c>
       <c r="Y1" s="17" t="s">
@@ -26693,9 +26712,9 @@
       <c r="P2" s="8" t="s">
         <v>78</v>
       </c>
-      <c r="Q2" s="36"/>
-      <c r="R2" s="36"/>
-      <c r="S2" s="36"/>
+      <c r="Q2" s="34"/>
+      <c r="R2" s="34"/>
+      <c r="S2" s="34"/>
       <c r="Y2" s="11">
         <f>B4</f>
         <v>46092</v>
@@ -27037,7 +27056,7 @@
       </c>
       <c r="B13" s="10">
         <f ca="1">IF(B11&lt;&gt;N3,(TODAY()-B12)*-1,"")</f>
-        <v>317</v>
+        <v>308</v>
       </c>
       <c r="D13" s="11"/>
       <c r="E13" s="15"/>
@@ -27550,21 +27569,21 @@
       <c r="K1" s="9" t="s">
         <v>42</v>
       </c>
-      <c r="M1" s="30" t="s">
-        <v>0</v>
-      </c>
-      <c r="N1" s="32"/>
-      <c r="O1" s="30" t="s">
+      <c r="M1" s="28" t="s">
+        <v>0</v>
+      </c>
+      <c r="N1" s="30"/>
+      <c r="O1" s="28" t="s">
         <v>5</v>
       </c>
-      <c r="P1" s="32"/>
-      <c r="Q1" s="35" t="s">
+      <c r="P1" s="30"/>
+      <c r="Q1" s="33" t="s">
         <v>79</v>
       </c>
-      <c r="R1" s="35" t="s">
+      <c r="R1" s="33" t="s">
         <v>45</v>
       </c>
-      <c r="S1" s="35" t="s">
+      <c r="S1" s="33" t="s">
         <v>84</v>
       </c>
       <c r="Y1" s="17" t="s">
@@ -27613,9 +27632,9 @@
       <c r="P2" s="8" t="s">
         <v>78</v>
       </c>
-      <c r="Q2" s="36"/>
-      <c r="R2" s="36"/>
-      <c r="S2" s="36"/>
+      <c r="Q2" s="34"/>
+      <c r="R2" s="34"/>
+      <c r="S2" s="34"/>
       <c r="Y2" s="11">
         <f>B4</f>
         <v>46091</v>
@@ -27679,7 +27698,7 @@
       </c>
       <c r="S3" s="2">
         <f ca="1">IF(COUNTIFS(D:D,"&lt;"&amp;TODAY(),J:J,"")=0,"",TODAY()-_xlfn.MINIFS(D:D,D:D,"&lt;"&amp;TODAY(),J:J,""))</f>
-        <v>29</v>
+        <v>38</v>
       </c>
       <c r="Y3" s="11">
         <f>J2</f>
@@ -27945,7 +27964,7 @@
       </c>
       <c r="B13" s="10">
         <f ca="1">IF(B11&lt;&gt;N3,(TODAY()-B12)*-1,"")</f>
-        <v>133</v>
+        <v>124</v>
       </c>
       <c r="D13" s="11"/>
       <c r="E13" s="15"/>
@@ -28461,21 +28480,21 @@
       <c r="K1" s="9" t="s">
         <v>42</v>
       </c>
-      <c r="M1" s="30" t="s">
-        <v>0</v>
-      </c>
-      <c r="N1" s="32"/>
-      <c r="O1" s="30" t="s">
+      <c r="M1" s="28" t="s">
+        <v>0</v>
+      </c>
+      <c r="N1" s="30"/>
+      <c r="O1" s="28" t="s">
         <v>5</v>
       </c>
-      <c r="P1" s="32"/>
-      <c r="Q1" s="35" t="s">
+      <c r="P1" s="30"/>
+      <c r="Q1" s="33" t="s">
         <v>79</v>
       </c>
-      <c r="R1" s="35" t="s">
+      <c r="R1" s="33" t="s">
         <v>45</v>
       </c>
-      <c r="S1" s="35" t="s">
+      <c r="S1" s="33" t="s">
         <v>84</v>
       </c>
       <c r="Y1" s="17" t="s">
@@ -28532,9 +28551,9 @@
       <c r="P2" s="8" t="s">
         <v>78</v>
       </c>
-      <c r="Q2" s="36"/>
-      <c r="R2" s="36"/>
-      <c r="S2" s="36"/>
+      <c r="Q2" s="34"/>
+      <c r="R2" s="34"/>
+      <c r="S2" s="34"/>
       <c r="Y2" s="11">
         <f>B4</f>
         <v>46073</v>
@@ -29381,21 +29400,21 @@
       <c r="K1" s="9" t="s">
         <v>42</v>
       </c>
-      <c r="M1" s="30" t="s">
-        <v>0</v>
-      </c>
-      <c r="N1" s="32"/>
-      <c r="O1" s="30" t="s">
+      <c r="M1" s="28" t="s">
+        <v>0</v>
+      </c>
+      <c r="N1" s="30"/>
+      <c r="O1" s="28" t="s">
         <v>5</v>
       </c>
-      <c r="P1" s="32"/>
-      <c r="Q1" s="35" t="s">
+      <c r="P1" s="30"/>
+      <c r="Q1" s="33" t="s">
         <v>79</v>
       </c>
-      <c r="R1" s="35" t="s">
+      <c r="R1" s="33" t="s">
         <v>45</v>
       </c>
-      <c r="S1" s="35" t="s">
+      <c r="S1" s="33" t="s">
         <v>84</v>
       </c>
       <c r="Y1" s="17" t="s">
@@ -29452,9 +29471,9 @@
       <c r="P2" s="8" t="s">
         <v>78</v>
       </c>
-      <c r="Q2" s="36"/>
-      <c r="R2" s="36"/>
-      <c r="S2" s="36"/>
+      <c r="Q2" s="34"/>
+      <c r="R2" s="34"/>
+      <c r="S2" s="34"/>
       <c r="Y2" s="11">
         <f>B4</f>
         <v>46073</v>
@@ -29784,7 +29803,7 @@
       </c>
       <c r="B13" s="10">
         <f ca="1">IF(B11&lt;&gt;N3,(TODAY()-B12)*-1,"")</f>
-        <v>114</v>
+        <v>105</v>
       </c>
       <c r="D13" s="11"/>
       <c r="E13" s="15"/>

</xml_diff>

<commit_message>
Dashboard update 2026-09-01 20:46
</commit_message>
<xml_diff>
--- a/excel/Crowdpear.xlsx
+++ b/excel/Crowdpear.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="30228"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="27932"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Investavimas 2026.06.03\Crowdpear\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="E:\Investavimas 2026.08.08\Crowdpear\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8B5D66E7-71A4-426B-A863-4C7DDD7F5D2C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F9EEFEA5-F194-4BD4-A1B9-42C74159CF85}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="17520" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Overview" sheetId="1" r:id="rId1"/>
@@ -601,6 +601,9 @@
     <xf numFmtId="2" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
+    <xf numFmtId="165" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
@@ -621,9 +624,6 @@
     </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="165" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="2">
@@ -3119,39 +3119,39 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:29" x14ac:dyDescent="0.25">
-      <c r="A1" s="28" t="s">
-        <v>0</v>
-      </c>
-      <c r="B1" s="29"/>
-      <c r="C1" s="29"/>
-      <c r="D1" s="29"/>
-      <c r="E1" s="29"/>
-      <c r="F1" s="29"/>
-      <c r="G1" s="30"/>
-      <c r="H1" s="31" t="s">
+      <c r="A1" s="29" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="30"/>
+      <c r="C1" s="30"/>
+      <c r="D1" s="30"/>
+      <c r="E1" s="30"/>
+      <c r="F1" s="30"/>
+      <c r="G1" s="31"/>
+      <c r="H1" s="32" t="s">
         <v>88</v>
       </c>
-      <c r="I1" s="31"/>
-      <c r="J1" s="31"/>
-      <c r="K1" s="31"/>
-      <c r="L1" s="31"/>
-      <c r="M1" s="31"/>
-      <c r="O1" s="31" t="s">
+      <c r="I1" s="32"/>
+      <c r="J1" s="32"/>
+      <c r="K1" s="32"/>
+      <c r="L1" s="32"/>
+      <c r="M1" s="32"/>
+      <c r="O1" s="32" t="s">
         <v>92</v>
       </c>
-      <c r="P1" s="31"/>
-      <c r="Q1" s="31"/>
-      <c r="R1" s="31"/>
-      <c r="S1" s="32" t="s">
+      <c r="P1" s="32"/>
+      <c r="Q1" s="32"/>
+      <c r="R1" s="32"/>
+      <c r="S1" s="33" t="s">
         <v>45</v>
       </c>
-      <c r="T1" s="32"/>
-      <c r="U1" s="32" t="s">
+      <c r="T1" s="33"/>
+      <c r="U1" s="33" t="s">
         <v>38</v>
       </c>
-      <c r="V1" s="32"/>
-      <c r="W1" s="32"/>
-      <c r="X1" s="32"/>
+      <c r="V1" s="33"/>
+      <c r="W1" s="33"/>
+      <c r="X1" s="33"/>
     </row>
     <row r="2" spans="1:29" x14ac:dyDescent="0.25">
       <c r="A2" s="6" t="s">
@@ -3293,7 +3293,7 @@
       </c>
       <c r="R3" s="4">
         <f>U3-P3</f>
-        <v>0</v>
+        <v>0.22000000000025466</v>
       </c>
       <c r="S3" s="4">
         <f>SUM(L3:L200)</f>
@@ -3301,23 +3301,23 @@
       </c>
       <c r="T3" s="4">
         <f>SUM(M3:M200)</f>
-        <v>116.47999999999999</v>
+        <v>116.69999999999999</v>
       </c>
       <c r="U3" s="4">
         <f>O3+T3+Q3</f>
-        <v>1186.48</v>
+        <v>1186.7</v>
       </c>
       <c r="V3" s="4">
         <f>U3-O3</f>
-        <v>156.48000000000002</v>
+        <v>156.70000000000005</v>
       </c>
       <c r="W3" s="14">
         <f>(U3-O3)/O3</f>
-        <v>0.15192233009708739</v>
+        <v>0.15213592233009712</v>
       </c>
       <c r="X3" s="14">
         <f ca="1">XIRR(Pinigai!K2:K200,Pinigai!A2:A200)</f>
-        <v>0.12784344553947447</v>
+        <v>0.12087267041206359</v>
       </c>
       <c r="AC3" s="4" t="str">
         <f ca="1">'Užnerio butai III'!AA2</f>
@@ -3818,7 +3818,7 @@
       </c>
       <c r="J12" s="10">
         <f ca="1">'Sfintii Arhangheli 21'!B13</f>
-        <v>33</v>
+        <v>9</v>
       </c>
       <c r="K12" s="10" t="str">
         <f ca="1">'Sfintii Arhangheli 21'!S3</f>
@@ -3932,7 +3932,7 @@
       </c>
       <c r="J14" s="10">
         <f ca="1">'Vienbutis Minsko 5A'!B13</f>
-        <v>40</v>
+        <v>16</v>
       </c>
       <c r="K14" s="10" t="str">
         <f ca="1">'Vienbutis Minsko 5A'!S3</f>
@@ -4046,7 +4046,7 @@
       </c>
       <c r="J16" s="10">
         <f ca="1">'Miškininkų 30 II'!B13</f>
-        <v>91</v>
+        <v>67</v>
       </c>
       <c r="K16" s="10" t="str">
         <f ca="1">'Miškininkų 30 II'!S3</f>
@@ -4058,7 +4058,7 @@
       </c>
       <c r="M16" s="4">
         <f>'Miškininkų 30 II'!P3</f>
-        <v>0.53</v>
+        <v>0.75</v>
       </c>
       <c r="AC16" s="4" t="str">
         <f ca="1">'Miškininkų 30 II'!AA2</f>
@@ -4103,7 +4103,7 @@
       </c>
       <c r="J17" s="10">
         <f ca="1">'Sūduvos 8-2'!B13</f>
-        <v>130</v>
+        <v>106</v>
       </c>
       <c r="K17" s="10" t="str">
         <f ca="1">'Sūduvos 8-2'!S3</f>
@@ -4160,7 +4160,7 @@
       </c>
       <c r="J18" s="10">
         <f ca="1">'Birelių namas II'!B13</f>
-        <v>137</v>
+        <v>113</v>
       </c>
       <c r="K18" s="10" t="str">
         <f ca="1">'Birelių namas II'!S3</f>
@@ -4274,7 +4274,7 @@
       </c>
       <c r="J20" s="10">
         <f ca="1">'Vingio namai XIV'!B13</f>
-        <v>179</v>
+        <v>155</v>
       </c>
       <c r="K20" s="10" t="str">
         <f ca="1">'Vingio namai XIV'!S3</f>
@@ -4388,7 +4388,7 @@
       </c>
       <c r="J22" s="10">
         <f ca="1">'Namas Panevėžyje'!B13</f>
-        <v>105</v>
+        <v>81</v>
       </c>
       <c r="K22" s="10" t="str">
         <f ca="1">'Namas Panevėžyje'!S3</f>
@@ -4502,11 +4502,11 @@
       </c>
       <c r="J24" s="10">
         <f ca="1">'Horizonto 2A XII'!B13</f>
-        <v>124</v>
+        <v>100</v>
       </c>
       <c r="K24" s="10">
         <f ca="1">'Horizonto 2A XII'!S3</f>
-        <v>38</v>
+        <v>62</v>
       </c>
       <c r="L24" s="4">
         <f>'Horizonto 2A XII'!N3</f>
@@ -4559,7 +4559,7 @@
       </c>
       <c r="J25" s="10">
         <f ca="1">'Tautvilo kotedžai XIV'!B13</f>
-        <v>308</v>
+        <v>284</v>
       </c>
       <c r="K25" s="10" t="str">
         <f ca="1">'Tautvilo kotedžai XIV'!S3</f>
@@ -4616,7 +4616,7 @@
       </c>
       <c r="J26" s="10">
         <f ca="1">'Kauno 36-118 II'!B13</f>
-        <v>221</v>
+        <v>197</v>
       </c>
       <c r="K26" s="10" t="str">
         <f ca="1">'Kauno 36-118 II'!S3</f>
@@ -4673,7 +4673,7 @@
       </c>
       <c r="J27" s="10">
         <f ca="1">'Vakaro 3A K1 III'!B13</f>
-        <v>336</v>
+        <v>312</v>
       </c>
       <c r="K27" s="10" t="str">
         <f ca="1">'Vakaro 3A K1 III'!S3</f>
@@ -4730,7 +4730,7 @@
       </c>
       <c r="J28" s="10">
         <f ca="1">'Užnerio butai XV'!B13</f>
-        <v>362</v>
+        <v>338</v>
       </c>
       <c r="K28" s="10" t="str">
         <f ca="1">'Užnerio butai XV'!S3</f>
@@ -4850,21 +4850,21 @@
       <c r="K1" s="9" t="s">
         <v>42</v>
       </c>
-      <c r="M1" s="28" t="s">
-        <v>0</v>
-      </c>
-      <c r="N1" s="30"/>
-      <c r="O1" s="28" t="s">
+      <c r="M1" s="29" t="s">
+        <v>0</v>
+      </c>
+      <c r="N1" s="31"/>
+      <c r="O1" s="29" t="s">
         <v>5</v>
       </c>
-      <c r="P1" s="30"/>
-      <c r="Q1" s="33" t="s">
+      <c r="P1" s="31"/>
+      <c r="Q1" s="34" t="s">
         <v>79</v>
       </c>
-      <c r="R1" s="33" t="s">
+      <c r="R1" s="34" t="s">
         <v>45</v>
       </c>
-      <c r="S1" s="33" t="s">
+      <c r="S1" s="34" t="s">
         <v>84</v>
       </c>
       <c r="Y1" s="17" t="s">
@@ -4921,9 +4921,9 @@
       <c r="P2" s="8" t="s">
         <v>78</v>
       </c>
-      <c r="Q2" s="34"/>
-      <c r="R2" s="34"/>
-      <c r="S2" s="34"/>
+      <c r="Q2" s="35"/>
+      <c r="R2" s="35"/>
+      <c r="S2" s="35"/>
       <c r="Y2" s="11">
         <f>B4</f>
         <v>46057</v>
@@ -5776,21 +5776,21 @@
       <c r="K1" s="9" t="s">
         <v>42</v>
       </c>
-      <c r="M1" s="28" t="s">
-        <v>0</v>
-      </c>
-      <c r="N1" s="30"/>
-      <c r="O1" s="28" t="s">
+      <c r="M1" s="29" t="s">
+        <v>0</v>
+      </c>
+      <c r="N1" s="31"/>
+      <c r="O1" s="29" t="s">
         <v>5</v>
       </c>
-      <c r="P1" s="30"/>
-      <c r="Q1" s="33" t="s">
+      <c r="P1" s="31"/>
+      <c r="Q1" s="34" t="s">
         <v>79</v>
       </c>
-      <c r="R1" s="33" t="s">
+      <c r="R1" s="34" t="s">
         <v>45</v>
       </c>
-      <c r="S1" s="33" t="s">
+      <c r="S1" s="34" t="s">
         <v>84</v>
       </c>
       <c r="Y1" s="17" t="s">
@@ -5847,9 +5847,9 @@
       <c r="P2" s="8" t="s">
         <v>78</v>
       </c>
-      <c r="Q2" s="34"/>
-      <c r="R2" s="34"/>
-      <c r="S2" s="34"/>
+      <c r="Q2" s="35"/>
+      <c r="R2" s="35"/>
+      <c r="S2" s="35"/>
       <c r="Y2" s="11">
         <f>B4</f>
         <v>46055</v>
@@ -6185,7 +6185,7 @@
       </c>
       <c r="B13" s="10">
         <f ca="1">IF(B11&lt;&gt;N3,(TODAY()-B12)*-1,"")</f>
-        <v>179</v>
+        <v>155</v>
       </c>
       <c r="D13" s="11"/>
       <c r="E13" s="15"/>
@@ -6701,21 +6701,21 @@
       <c r="K1" s="9" t="s">
         <v>42</v>
       </c>
-      <c r="M1" s="28" t="s">
-        <v>0</v>
-      </c>
-      <c r="N1" s="30"/>
-      <c r="O1" s="28" t="s">
+      <c r="M1" s="29" t="s">
+        <v>0</v>
+      </c>
+      <c r="N1" s="31"/>
+      <c r="O1" s="29" t="s">
         <v>5</v>
       </c>
-      <c r="P1" s="30"/>
-      <c r="Q1" s="33" t="s">
+      <c r="P1" s="31"/>
+      <c r="Q1" s="34" t="s">
         <v>79</v>
       </c>
-      <c r="R1" s="33" t="s">
+      <c r="R1" s="34" t="s">
         <v>45</v>
       </c>
-      <c r="S1" s="33" t="s">
+      <c r="S1" s="34" t="s">
         <v>84</v>
       </c>
       <c r="Y1" s="17" t="s">
@@ -6772,9 +6772,9 @@
       <c r="P2" s="8" t="s">
         <v>78</v>
       </c>
-      <c r="Q2" s="34"/>
-      <c r="R2" s="34"/>
-      <c r="S2" s="34"/>
+      <c r="Q2" s="35"/>
+      <c r="R2" s="35"/>
+      <c r="S2" s="35"/>
       <c r="Y2" s="11">
         <f>B4</f>
         <v>46043</v>
@@ -7649,21 +7649,21 @@
       <c r="K1" s="9" t="s">
         <v>42</v>
       </c>
-      <c r="M1" s="28" t="s">
-        <v>0</v>
-      </c>
-      <c r="N1" s="30"/>
-      <c r="O1" s="28" t="s">
+      <c r="M1" s="29" t="s">
+        <v>0</v>
+      </c>
+      <c r="N1" s="31"/>
+      <c r="O1" s="29" t="s">
         <v>5</v>
       </c>
-      <c r="P1" s="30"/>
-      <c r="Q1" s="33" t="s">
+      <c r="P1" s="31"/>
+      <c r="Q1" s="34" t="s">
         <v>79</v>
       </c>
-      <c r="R1" s="33" t="s">
+      <c r="R1" s="34" t="s">
         <v>45</v>
       </c>
-      <c r="S1" s="33" t="s">
+      <c r="S1" s="34" t="s">
         <v>84</v>
       </c>
       <c r="Y1" s="17" t="s">
@@ -7720,9 +7720,9 @@
       <c r="P2" s="8" t="s">
         <v>78</v>
       </c>
-      <c r="Q2" s="34"/>
-      <c r="R2" s="34"/>
-      <c r="S2" s="34"/>
+      <c r="Q2" s="35"/>
+      <c r="R2" s="35"/>
+      <c r="S2" s="35"/>
       <c r="Y2" s="11">
         <f>B4</f>
         <v>46013</v>
@@ -8066,7 +8066,7 @@
       </c>
       <c r="B13" s="10">
         <f ca="1">IF(B11&lt;&gt;N3,(TODAY()-B12)*-1,"")</f>
-        <v>137</v>
+        <v>113</v>
       </c>
       <c r="D13" s="11"/>
       <c r="E13" s="15"/>
@@ -8579,21 +8579,21 @@
       <c r="K1" s="9" t="s">
         <v>42</v>
       </c>
-      <c r="M1" s="28" t="s">
-        <v>0</v>
-      </c>
-      <c r="N1" s="30"/>
-      <c r="O1" s="28" t="s">
+      <c r="M1" s="29" t="s">
+        <v>0</v>
+      </c>
+      <c r="N1" s="31"/>
+      <c r="O1" s="29" t="s">
         <v>5</v>
       </c>
-      <c r="P1" s="30"/>
-      <c r="Q1" s="33" t="s">
+      <c r="P1" s="31"/>
+      <c r="Q1" s="34" t="s">
         <v>79</v>
       </c>
-      <c r="R1" s="33" t="s">
+      <c r="R1" s="34" t="s">
         <v>45</v>
       </c>
-      <c r="S1" s="33" t="s">
+      <c r="S1" s="34" t="s">
         <v>84</v>
       </c>
       <c r="Y1" s="17" t="s">
@@ -8650,9 +8650,9 @@
       <c r="P2" s="8" t="s">
         <v>78</v>
       </c>
-      <c r="Q2" s="34"/>
-      <c r="R2" s="34"/>
-      <c r="S2" s="34"/>
+      <c r="Q2" s="35"/>
+      <c r="R2" s="35"/>
+      <c r="S2" s="35"/>
       <c r="Y2" s="11">
         <f>B4</f>
         <v>46003</v>
@@ -8996,7 +8996,7 @@
       </c>
       <c r="B13" s="10">
         <f ca="1">IF(B11&lt;&gt;N3,(TODAY()-B12)*-1,"")</f>
-        <v>130</v>
+        <v>106</v>
       </c>
       <c r="D13" s="11"/>
       <c r="E13" s="15"/>
@@ -9509,21 +9509,21 @@
       <c r="K1" s="9" t="s">
         <v>42</v>
       </c>
-      <c r="M1" s="28" t="s">
-        <v>0</v>
-      </c>
-      <c r="N1" s="30"/>
-      <c r="O1" s="28" t="s">
+      <c r="M1" s="29" t="s">
+        <v>0</v>
+      </c>
+      <c r="N1" s="31"/>
+      <c r="O1" s="29" t="s">
         <v>5</v>
       </c>
-      <c r="P1" s="30"/>
-      <c r="Q1" s="33" t="s">
+      <c r="P1" s="31"/>
+      <c r="Q1" s="34" t="s">
         <v>79</v>
       </c>
-      <c r="R1" s="33" t="s">
+      <c r="R1" s="34" t="s">
         <v>45</v>
       </c>
-      <c r="S1" s="33" t="s">
+      <c r="S1" s="34" t="s">
         <v>84</v>
       </c>
       <c r="Y1" s="17" t="s">
@@ -9580,9 +9580,9 @@
       <c r="P2" s="8" t="s">
         <v>78</v>
       </c>
-      <c r="Q2" s="34"/>
-      <c r="R2" s="34"/>
-      <c r="S2" s="34"/>
+      <c r="Q2" s="35"/>
+      <c r="R2" s="35"/>
+      <c r="S2" s="35"/>
       <c r="Y2" s="11">
         <f>B4</f>
         <v>45967</v>
@@ -9642,7 +9642,7 @@
       </c>
       <c r="P3" s="4">
         <f>H42+I42</f>
-        <v>0.53</v>
+        <v>0.75</v>
       </c>
       <c r="Q3" s="14" t="str">
         <f>IF(M3=N3,XIRR(Z2:Z14,Y2:Y14),"")</f>
@@ -9681,13 +9681,21 @@
       <c r="F4" s="4">
         <v>0.22</v>
       </c>
-      <c r="G4" s="4"/>
-      <c r="H4" s="4"/>
-      <c r="I4" s="4"/>
-      <c r="J4" s="11"/>
-      <c r="K4" s="10" t="str">
-        <f t="shared" si="0"/>
-        <v/>
+      <c r="G4" s="4">
+        <v>0</v>
+      </c>
+      <c r="H4" s="4">
+        <v>0.22</v>
+      </c>
+      <c r="I4" s="4">
+        <v>0</v>
+      </c>
+      <c r="J4" s="11">
+        <v>46265</v>
+      </c>
+      <c r="K4" s="10">
+        <f t="shared" si="0"/>
+        <v>0</v>
       </c>
       <c r="Y4" s="11">
         <f t="shared" ref="Y4:Y14" si="1">J3</f>
@@ -9724,11 +9732,11 @@
       </c>
       <c r="Y5" s="11">
         <f t="shared" si="1"/>
-        <v>0</v>
+        <v>46265</v>
       </c>
       <c r="Z5" s="4">
         <f t="shared" si="2"/>
-        <v>0</v>
+        <v>0.22</v>
       </c>
     </row>
     <row r="6" spans="1:27" x14ac:dyDescent="0.25">
@@ -9926,7 +9934,7 @@
       </c>
       <c r="B13" s="10">
         <f ca="1">IF(B11&lt;&gt;N3,(TODAY()-B12)*-1,"")</f>
-        <v>91</v>
+        <v>67</v>
       </c>
       <c r="D13" s="11"/>
       <c r="E13" s="15"/>
@@ -10349,7 +10357,7 @@
       </c>
       <c r="H42" s="4">
         <f t="shared" si="3"/>
-        <v>0.53</v>
+        <v>0.75</v>
       </c>
       <c r="I42" s="4">
         <f t="shared" si="3"/>
@@ -10442,21 +10450,21 @@
       <c r="K1" s="9" t="s">
         <v>42</v>
       </c>
-      <c r="M1" s="28" t="s">
-        <v>0</v>
-      </c>
-      <c r="N1" s="30"/>
-      <c r="O1" s="28" t="s">
+      <c r="M1" s="29" t="s">
+        <v>0</v>
+      </c>
+      <c r="N1" s="31"/>
+      <c r="O1" s="29" t="s">
         <v>5</v>
       </c>
-      <c r="P1" s="30"/>
-      <c r="Q1" s="33" t="s">
+      <c r="P1" s="31"/>
+      <c r="Q1" s="34" t="s">
         <v>79</v>
       </c>
-      <c r="R1" s="33" t="s">
+      <c r="R1" s="34" t="s">
         <v>45</v>
       </c>
-      <c r="S1" s="33" t="s">
+      <c r="S1" s="34" t="s">
         <v>84</v>
       </c>
       <c r="Y1" s="17" t="s">
@@ -10513,9 +10521,9 @@
       <c r="P2" s="8" t="s">
         <v>78</v>
       </c>
-      <c r="Q2" s="34"/>
-      <c r="R2" s="34"/>
-      <c r="S2" s="34"/>
+      <c r="Q2" s="35"/>
+      <c r="R2" s="35"/>
+      <c r="S2" s="35"/>
       <c r="Y2" s="11">
         <f>B4</f>
         <v>45951</v>
@@ -11376,21 +11384,21 @@
       <c r="K1" s="9" t="s">
         <v>42</v>
       </c>
-      <c r="M1" s="28" t="s">
-        <v>0</v>
-      </c>
-      <c r="N1" s="30"/>
-      <c r="O1" s="28" t="s">
+      <c r="M1" s="29" t="s">
+        <v>0</v>
+      </c>
+      <c r="N1" s="31"/>
+      <c r="O1" s="29" t="s">
         <v>5</v>
       </c>
-      <c r="P1" s="30"/>
-      <c r="Q1" s="33" t="s">
+      <c r="P1" s="31"/>
+      <c r="Q1" s="34" t="s">
         <v>79</v>
       </c>
-      <c r="R1" s="33" t="s">
+      <c r="R1" s="34" t="s">
         <v>45</v>
       </c>
-      <c r="S1" s="33" t="s">
+      <c r="S1" s="34" t="s">
         <v>84</v>
       </c>
       <c r="Y1" s="17" t="s">
@@ -11447,9 +11455,9 @@
       <c r="P2" s="8" t="s">
         <v>78</v>
       </c>
-      <c r="Q2" s="34"/>
-      <c r="R2" s="34"/>
-      <c r="S2" s="34"/>
+      <c r="Q2" s="35"/>
+      <c r="R2" s="35"/>
+      <c r="S2" s="35"/>
       <c r="Y2" s="11">
         <f>B4</f>
         <v>45916</v>
@@ -11801,7 +11809,7 @@
       </c>
       <c r="B13" s="10">
         <f ca="1">IF(B11&lt;&gt;N3,(TODAY()-B12)*-1,"")</f>
-        <v>40</v>
+        <v>16</v>
       </c>
       <c r="D13" s="11"/>
       <c r="E13" s="15"/>
@@ -12317,21 +12325,21 @@
       <c r="K1" s="9" t="s">
         <v>42</v>
       </c>
-      <c r="M1" s="28" t="s">
-        <v>0</v>
-      </c>
-      <c r="N1" s="30"/>
-      <c r="O1" s="28" t="s">
+      <c r="M1" s="29" t="s">
+        <v>0</v>
+      </c>
+      <c r="N1" s="31"/>
+      <c r="O1" s="29" t="s">
         <v>5</v>
       </c>
-      <c r="P1" s="30"/>
-      <c r="Q1" s="33" t="s">
+      <c r="P1" s="31"/>
+      <c r="Q1" s="34" t="s">
         <v>79</v>
       </c>
-      <c r="R1" s="33" t="s">
+      <c r="R1" s="34" t="s">
         <v>45</v>
       </c>
-      <c r="S1" s="33" t="s">
+      <c r="S1" s="34" t="s">
         <v>84</v>
       </c>
       <c r="Y1" s="17" t="s">
@@ -12388,9 +12396,9 @@
       <c r="P2" s="8" t="s">
         <v>78</v>
       </c>
-      <c r="Q2" s="34"/>
-      <c r="R2" s="34"/>
-      <c r="S2" s="34"/>
+      <c r="Q2" s="35"/>
+      <c r="R2" s="35"/>
+      <c r="S2" s="35"/>
       <c r="Y2" s="11">
         <f>B4</f>
         <v>45917</v>
@@ -13251,21 +13259,21 @@
       <c r="K1" s="9" t="s">
         <v>42</v>
       </c>
-      <c r="M1" s="28" t="s">
-        <v>0</v>
-      </c>
-      <c r="N1" s="30"/>
-      <c r="O1" s="28" t="s">
+      <c r="M1" s="29" t="s">
+        <v>0</v>
+      </c>
+      <c r="N1" s="31"/>
+      <c r="O1" s="29" t="s">
         <v>5</v>
       </c>
-      <c r="P1" s="30"/>
-      <c r="Q1" s="33" t="s">
+      <c r="P1" s="31"/>
+      <c r="Q1" s="34" t="s">
         <v>79</v>
       </c>
-      <c r="R1" s="33" t="s">
+      <c r="R1" s="34" t="s">
         <v>45</v>
       </c>
-      <c r="S1" s="33" t="s">
+      <c r="S1" s="34" t="s">
         <v>84</v>
       </c>
       <c r="Y1" s="17" t="s">
@@ -13322,9 +13330,9 @@
       <c r="P2" s="8" t="s">
         <v>78</v>
       </c>
-      <c r="Q2" s="34"/>
-      <c r="R2" s="34"/>
-      <c r="S2" s="34"/>
+      <c r="Q2" s="35"/>
+      <c r="R2" s="35"/>
+      <c r="S2" s="35"/>
       <c r="Y2" s="11">
         <f>B4</f>
         <v>45908</v>
@@ -13676,7 +13684,7 @@
       </c>
       <c r="B13" s="10">
         <f ca="1">IF(B11&lt;&gt;N3,(TODAY()-B12)*-1,"")</f>
-        <v>33</v>
+        <v>9</v>
       </c>
       <c r="D13" s="11"/>
       <c r="E13" s="15"/>
@@ -14460,11 +14468,11 @@
     <row r="200" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A200" s="12">
         <f ca="1">TODAY()</f>
-        <v>46241</v>
+        <v>46265</v>
       </c>
       <c r="K200" s="25">
         <f>Overview!U3</f>
-        <v>1186.48</v>
+        <v>1186.7</v>
       </c>
     </row>
   </sheetData>
@@ -14526,21 +14534,21 @@
       <c r="K1" s="9" t="s">
         <v>42</v>
       </c>
-      <c r="M1" s="28" t="s">
-        <v>0</v>
-      </c>
-      <c r="N1" s="30"/>
-      <c r="O1" s="28" t="s">
+      <c r="M1" s="29" t="s">
+        <v>0</v>
+      </c>
+      <c r="N1" s="31"/>
+      <c r="O1" s="29" t="s">
         <v>5</v>
       </c>
-      <c r="P1" s="30"/>
-      <c r="Q1" s="33" t="s">
+      <c r="P1" s="31"/>
+      <c r="Q1" s="34" t="s">
         <v>79</v>
       </c>
-      <c r="R1" s="33" t="s">
+      <c r="R1" s="34" t="s">
         <v>45</v>
       </c>
-      <c r="S1" s="33" t="s">
+      <c r="S1" s="34" t="s">
         <v>84</v>
       </c>
       <c r="Y1" s="17" t="s">
@@ -14597,9 +14605,9 @@
       <c r="P2" s="8" t="s">
         <v>78</v>
       </c>
-      <c r="Q2" s="34"/>
-      <c r="R2" s="34"/>
-      <c r="S2" s="34"/>
+      <c r="Q2" s="35"/>
+      <c r="R2" s="35"/>
+      <c r="S2" s="35"/>
       <c r="Y2" s="11">
         <f>B3</f>
         <v>45791</v>
@@ -15449,21 +15457,21 @@
       <c r="K1" s="9" t="s">
         <v>42</v>
       </c>
-      <c r="M1" s="28" t="s">
-        <v>0</v>
-      </c>
-      <c r="N1" s="30"/>
-      <c r="O1" s="28" t="s">
+      <c r="M1" s="29" t="s">
+        <v>0</v>
+      </c>
+      <c r="N1" s="31"/>
+      <c r="O1" s="29" t="s">
         <v>5</v>
       </c>
-      <c r="P1" s="30"/>
-      <c r="Q1" s="33" t="s">
+      <c r="P1" s="31"/>
+      <c r="Q1" s="34" t="s">
         <v>79</v>
       </c>
-      <c r="R1" s="33" t="s">
+      <c r="R1" s="34" t="s">
         <v>45</v>
       </c>
-      <c r="S1" s="33" t="s">
+      <c r="S1" s="34" t="s">
         <v>84</v>
       </c>
       <c r="Y1" s="17" t="s">
@@ -15520,9 +15528,9 @@
       <c r="P2" s="8" t="s">
         <v>78</v>
       </c>
-      <c r="Q2" s="34"/>
-      <c r="R2" s="34"/>
-      <c r="S2" s="34"/>
+      <c r="Q2" s="35"/>
+      <c r="R2" s="35"/>
+      <c r="S2" s="35"/>
       <c r="Y2" s="11">
         <f>B3</f>
         <v>45770</v>
@@ -16400,21 +16408,21 @@
       <c r="K1" s="9" t="s">
         <v>42</v>
       </c>
-      <c r="M1" s="28" t="s">
-        <v>0</v>
-      </c>
-      <c r="N1" s="30"/>
-      <c r="O1" s="28" t="s">
+      <c r="M1" s="29" t="s">
+        <v>0</v>
+      </c>
+      <c r="N1" s="31"/>
+      <c r="O1" s="29" t="s">
         <v>5</v>
       </c>
-      <c r="P1" s="30"/>
-      <c r="Q1" s="33" t="s">
+      <c r="P1" s="31"/>
+      <c r="Q1" s="34" t="s">
         <v>79</v>
       </c>
-      <c r="R1" s="33" t="s">
+      <c r="R1" s="34" t="s">
         <v>45</v>
       </c>
-      <c r="S1" s="33" t="s">
+      <c r="S1" s="34" t="s">
         <v>84</v>
       </c>
       <c r="Y1" s="17" t="s">
@@ -16471,9 +16479,9 @@
       <c r="P2" s="8" t="s">
         <v>78</v>
       </c>
-      <c r="Q2" s="34"/>
-      <c r="R2" s="34"/>
-      <c r="S2" s="34"/>
+      <c r="Q2" s="35"/>
+      <c r="R2" s="35"/>
+      <c r="S2" s="35"/>
       <c r="Y2" s="11">
         <f>B3</f>
         <v>45764</v>
@@ -17365,21 +17373,21 @@
       <c r="K1" s="9" t="s">
         <v>42</v>
       </c>
-      <c r="M1" s="28" t="s">
-        <v>0</v>
-      </c>
-      <c r="N1" s="30"/>
-      <c r="O1" s="28" t="s">
+      <c r="M1" s="29" t="s">
+        <v>0</v>
+      </c>
+      <c r="N1" s="31"/>
+      <c r="O1" s="29" t="s">
         <v>5</v>
       </c>
-      <c r="P1" s="30"/>
-      <c r="Q1" s="33" t="s">
+      <c r="P1" s="31"/>
+      <c r="Q1" s="34" t="s">
         <v>79</v>
       </c>
-      <c r="R1" s="33" t="s">
+      <c r="R1" s="34" t="s">
         <v>45</v>
       </c>
-      <c r="S1" s="33" t="s">
+      <c r="S1" s="34" t="s">
         <v>84</v>
       </c>
       <c r="Y1" s="17" t="s">
@@ -17436,9 +17444,9 @@
       <c r="P2" s="8" t="s">
         <v>78</v>
       </c>
-      <c r="Q2" s="34"/>
-      <c r="R2" s="34"/>
-      <c r="S2" s="34"/>
+      <c r="Q2" s="35"/>
+      <c r="R2" s="35"/>
+      <c r="S2" s="35"/>
       <c r="Y2" s="11">
         <f>B3</f>
         <v>45757</v>
@@ -18287,21 +18295,21 @@
       <c r="K1" s="9" t="s">
         <v>42</v>
       </c>
-      <c r="M1" s="28" t="s">
-        <v>0</v>
-      </c>
-      <c r="N1" s="30"/>
-      <c r="O1" s="28" t="s">
+      <c r="M1" s="29" t="s">
+        <v>0</v>
+      </c>
+      <c r="N1" s="31"/>
+      <c r="O1" s="29" t="s">
         <v>5</v>
       </c>
-      <c r="P1" s="30"/>
-      <c r="Q1" s="33" t="s">
+      <c r="P1" s="31"/>
+      <c r="Q1" s="34" t="s">
         <v>79</v>
       </c>
-      <c r="R1" s="33" t="s">
+      <c r="R1" s="34" t="s">
         <v>45</v>
       </c>
-      <c r="S1" s="33" t="s">
+      <c r="S1" s="34" t="s">
         <v>84</v>
       </c>
       <c r="Y1" s="17" t="s">
@@ -18358,9 +18366,9 @@
       <c r="P2" s="8" t="s">
         <v>78</v>
       </c>
-      <c r="Q2" s="34"/>
-      <c r="R2" s="34"/>
-      <c r="S2" s="34"/>
+      <c r="Q2" s="35"/>
+      <c r="R2" s="35"/>
+      <c r="S2" s="35"/>
       <c r="Y2" s="11">
         <f>B3</f>
         <v>45743</v>
@@ -19251,21 +19259,21 @@
       <c r="K1" s="9" t="s">
         <v>42</v>
       </c>
-      <c r="M1" s="28" t="s">
-        <v>0</v>
-      </c>
-      <c r="N1" s="30"/>
-      <c r="O1" s="28" t="s">
+      <c r="M1" s="29" t="s">
+        <v>0</v>
+      </c>
+      <c r="N1" s="31"/>
+      <c r="O1" s="29" t="s">
         <v>5</v>
       </c>
-      <c r="P1" s="30"/>
-      <c r="Q1" s="33" t="s">
+      <c r="P1" s="31"/>
+      <c r="Q1" s="34" t="s">
         <v>79</v>
       </c>
-      <c r="R1" s="33" t="s">
+      <c r="R1" s="34" t="s">
         <v>45</v>
       </c>
-      <c r="S1" s="33" t="s">
+      <c r="S1" s="34" t="s">
         <v>84</v>
       </c>
       <c r="Y1" s="17" t="s">
@@ -19322,9 +19330,9 @@
       <c r="P2" s="8" t="s">
         <v>78</v>
       </c>
-      <c r="Q2" s="34"/>
-      <c r="R2" s="34"/>
-      <c r="S2" s="34"/>
+      <c r="Q2" s="35"/>
+      <c r="R2" s="35"/>
+      <c r="S2" s="35"/>
       <c r="Y2" s="11">
         <f>B3</f>
         <v>45729</v>
@@ -20403,21 +20411,21 @@
       <c r="K1" s="9" t="s">
         <v>42</v>
       </c>
-      <c r="M1" s="28" t="s">
-        <v>0</v>
-      </c>
-      <c r="N1" s="30"/>
-      <c r="O1" s="28" t="s">
+      <c r="M1" s="29" t="s">
+        <v>0</v>
+      </c>
+      <c r="N1" s="31"/>
+      <c r="O1" s="29" t="s">
         <v>5</v>
       </c>
-      <c r="P1" s="30"/>
-      <c r="Q1" s="33" t="s">
+      <c r="P1" s="31"/>
+      <c r="Q1" s="34" t="s">
         <v>79</v>
       </c>
-      <c r="R1" s="33" t="s">
+      <c r="R1" s="34" t="s">
         <v>45</v>
       </c>
-      <c r="S1" s="33" t="s">
+      <c r="S1" s="34" t="s">
         <v>84</v>
       </c>
       <c r="Y1" s="17" t="s">
@@ -20474,9 +20482,9 @@
       <c r="P2" s="8" t="s">
         <v>78</v>
       </c>
-      <c r="Q2" s="34"/>
-      <c r="R2" s="34"/>
-      <c r="S2" s="34"/>
+      <c r="Q2" s="35"/>
+      <c r="R2" s="35"/>
+      <c r="S2" s="35"/>
       <c r="Y2" s="11">
         <f>B3</f>
         <v>45725</v>
@@ -21556,21 +21564,21 @@
       <c r="K1" s="9" t="s">
         <v>42</v>
       </c>
-      <c r="M1" s="28" t="s">
-        <v>0</v>
-      </c>
-      <c r="N1" s="30"/>
-      <c r="O1" s="28" t="s">
+      <c r="M1" s="29" t="s">
+        <v>0</v>
+      </c>
+      <c r="N1" s="31"/>
+      <c r="O1" s="29" t="s">
         <v>5</v>
       </c>
-      <c r="P1" s="30"/>
-      <c r="Q1" s="33" t="s">
+      <c r="P1" s="31"/>
+      <c r="Q1" s="34" t="s">
         <v>79</v>
       </c>
-      <c r="R1" s="33" t="s">
+      <c r="R1" s="34" t="s">
         <v>45</v>
       </c>
-      <c r="S1" s="33" t="s">
+      <c r="S1" s="34" t="s">
         <v>84</v>
       </c>
       <c r="Y1" s="17" t="s">
@@ -21627,9 +21635,9 @@
       <c r="P2" s="8" t="s">
         <v>78</v>
       </c>
-      <c r="Q2" s="34"/>
-      <c r="R2" s="34"/>
-      <c r="S2" s="34"/>
+      <c r="Q2" s="35"/>
+      <c r="R2" s="35"/>
+      <c r="S2" s="35"/>
       <c r="Y2" s="11">
         <f>B3</f>
         <v>45721</v>
@@ -22725,21 +22733,21 @@
       <c r="K1" s="9" t="s">
         <v>42</v>
       </c>
-      <c r="M1" s="28" t="s">
-        <v>0</v>
-      </c>
-      <c r="N1" s="30"/>
-      <c r="O1" s="28" t="s">
+      <c r="M1" s="29" t="s">
+        <v>0</v>
+      </c>
+      <c r="N1" s="31"/>
+      <c r="O1" s="29" t="s">
         <v>5</v>
       </c>
-      <c r="P1" s="30"/>
-      <c r="Q1" s="33" t="s">
+      <c r="P1" s="31"/>
+      <c r="Q1" s="34" t="s">
         <v>79</v>
       </c>
-      <c r="R1" s="33" t="s">
+      <c r="R1" s="34" t="s">
         <v>45</v>
       </c>
-      <c r="S1" s="33" t="s">
+      <c r="S1" s="34" t="s">
         <v>84</v>
       </c>
       <c r="Y1" s="17" t="s">
@@ -22796,9 +22804,9 @@
       <c r="P2" s="8" t="s">
         <v>78</v>
       </c>
-      <c r="Q2" s="34"/>
-      <c r="R2" s="34"/>
-      <c r="S2" s="34"/>
+      <c r="Q2" s="35"/>
+      <c r="R2" s="35"/>
+      <c r="S2" s="35"/>
       <c r="Y2" s="11">
         <f>B3</f>
         <v>45719</v>
@@ -23891,21 +23899,21 @@
       <c r="K1" s="9" t="s">
         <v>42</v>
       </c>
-      <c r="M1" s="28" t="s">
-        <v>0</v>
-      </c>
-      <c r="N1" s="30"/>
-      <c r="O1" s="28" t="s">
+      <c r="M1" s="29" t="s">
+        <v>0</v>
+      </c>
+      <c r="N1" s="31"/>
+      <c r="O1" s="29" t="s">
         <v>5</v>
       </c>
-      <c r="P1" s="30"/>
-      <c r="Q1" s="33" t="s">
+      <c r="P1" s="31"/>
+      <c r="Q1" s="34" t="s">
         <v>79</v>
       </c>
-      <c r="R1" s="33" t="s">
+      <c r="R1" s="34" t="s">
         <v>45</v>
       </c>
-      <c r="S1" s="33" t="s">
+      <c r="S1" s="34" t="s">
         <v>84</v>
       </c>
       <c r="Y1" s="17" t="s">
@@ -23954,9 +23962,9 @@
       <c r="P2" s="8" t="s">
         <v>78</v>
       </c>
-      <c r="Q2" s="34"/>
-      <c r="R2" s="34"/>
-      <c r="S2" s="34"/>
+      <c r="Q2" s="35"/>
+      <c r="R2" s="35"/>
+      <c r="S2" s="35"/>
       <c r="Y2" s="11">
         <f>B4</f>
         <v>46238</v>
@@ -24263,7 +24271,7 @@
       <c r="A12" s="7" t="s">
         <v>85</v>
       </c>
-      <c r="B12" s="35">
+      <c r="B12" s="28">
         <v>46603</v>
       </c>
       <c r="D12" s="11"/>
@@ -24292,7 +24300,7 @@
       </c>
       <c r="B13" s="10">
         <f ca="1">IF(B11&lt;&gt;N3,(TODAY()-B12)*-1,"")</f>
-        <v>362</v>
+        <v>338</v>
       </c>
       <c r="D13" s="11"/>
       <c r="E13" s="4"/>
@@ -24805,21 +24813,21 @@
       <c r="K1" s="9" t="s">
         <v>42</v>
       </c>
-      <c r="M1" s="28" t="s">
-        <v>0</v>
-      </c>
-      <c r="N1" s="30"/>
-      <c r="O1" s="28" t="s">
+      <c r="M1" s="29" t="s">
+        <v>0</v>
+      </c>
+      <c r="N1" s="31"/>
+      <c r="O1" s="29" t="s">
         <v>5</v>
       </c>
-      <c r="P1" s="30"/>
-      <c r="Q1" s="33" t="s">
+      <c r="P1" s="31"/>
+      <c r="Q1" s="34" t="s">
         <v>79</v>
       </c>
-      <c r="R1" s="33" t="s">
+      <c r="R1" s="34" t="s">
         <v>45</v>
       </c>
-      <c r="S1" s="33" t="s">
+      <c r="S1" s="34" t="s">
         <v>84</v>
       </c>
       <c r="Y1" s="17" t="s">
@@ -24868,9 +24876,9 @@
       <c r="P2" s="8" t="s">
         <v>78</v>
       </c>
-      <c r="Q2" s="34"/>
-      <c r="R2" s="34"/>
-      <c r="S2" s="34"/>
+      <c r="Q2" s="35"/>
+      <c r="R2" s="35"/>
+      <c r="S2" s="35"/>
       <c r="Y2" s="11">
         <f>B4</f>
         <v>46212</v>
@@ -25206,7 +25214,7 @@
       </c>
       <c r="B13" s="10">
         <f ca="1">IF(B11&lt;&gt;N3,(TODAY()-B12)*-1,"")</f>
-        <v>336</v>
+        <v>312</v>
       </c>
       <c r="D13" s="11"/>
       <c r="E13" s="15"/>
@@ -25719,21 +25727,21 @@
       <c r="K1" s="9" t="s">
         <v>42</v>
       </c>
-      <c r="M1" s="28" t="s">
-        <v>0</v>
-      </c>
-      <c r="N1" s="30"/>
-      <c r="O1" s="28" t="s">
+      <c r="M1" s="29" t="s">
+        <v>0</v>
+      </c>
+      <c r="N1" s="31"/>
+      <c r="O1" s="29" t="s">
         <v>5</v>
       </c>
-      <c r="P1" s="30"/>
-      <c r="Q1" s="33" t="s">
+      <c r="P1" s="31"/>
+      <c r="Q1" s="34" t="s">
         <v>79</v>
       </c>
-      <c r="R1" s="33" t="s">
+      <c r="R1" s="34" t="s">
         <v>45</v>
       </c>
-      <c r="S1" s="33" t="s">
+      <c r="S1" s="34" t="s">
         <v>84</v>
       </c>
       <c r="Y1" s="17" t="s">
@@ -25790,9 +25798,9 @@
       <c r="P2" s="8" t="s">
         <v>78</v>
       </c>
-      <c r="Q2" s="34"/>
-      <c r="R2" s="34"/>
-      <c r="S2" s="34"/>
+      <c r="Q2" s="35"/>
+      <c r="R2" s="35"/>
+      <c r="S2" s="35"/>
       <c r="Y2" s="11">
         <f>B4</f>
         <v>46097</v>
@@ -26128,7 +26136,7 @@
       </c>
       <c r="B13" s="10">
         <f ca="1">IF(B11&lt;&gt;N3,(TODAY()-B12)*-1,"")</f>
-        <v>221</v>
+        <v>197</v>
       </c>
       <c r="D13" s="11"/>
       <c r="E13" s="15"/>
@@ -26641,21 +26649,21 @@
       <c r="K1" s="9" t="s">
         <v>42</v>
       </c>
-      <c r="M1" s="28" t="s">
-        <v>0</v>
-      </c>
-      <c r="N1" s="30"/>
-      <c r="O1" s="28" t="s">
+      <c r="M1" s="29" t="s">
+        <v>0</v>
+      </c>
+      <c r="N1" s="31"/>
+      <c r="O1" s="29" t="s">
         <v>5</v>
       </c>
-      <c r="P1" s="30"/>
-      <c r="Q1" s="33" t="s">
+      <c r="P1" s="31"/>
+      <c r="Q1" s="34" t="s">
         <v>79</v>
       </c>
-      <c r="R1" s="33" t="s">
+      <c r="R1" s="34" t="s">
         <v>45</v>
       </c>
-      <c r="S1" s="33" t="s">
+      <c r="S1" s="34" t="s">
         <v>84</v>
       </c>
       <c r="Y1" s="17" t="s">
@@ -26712,9 +26720,9 @@
       <c r="P2" s="8" t="s">
         <v>78</v>
       </c>
-      <c r="Q2" s="34"/>
-      <c r="R2" s="34"/>
-      <c r="S2" s="34"/>
+      <c r="Q2" s="35"/>
+      <c r="R2" s="35"/>
+      <c r="S2" s="35"/>
       <c r="Y2" s="11">
         <f>B4</f>
         <v>46092</v>
@@ -27056,7 +27064,7 @@
       </c>
       <c r="B13" s="10">
         <f ca="1">IF(B11&lt;&gt;N3,(TODAY()-B12)*-1,"")</f>
-        <v>308</v>
+        <v>284</v>
       </c>
       <c r="D13" s="11"/>
       <c r="E13" s="15"/>
@@ -27569,21 +27577,21 @@
       <c r="K1" s="9" t="s">
         <v>42</v>
       </c>
-      <c r="M1" s="28" t="s">
-        <v>0</v>
-      </c>
-      <c r="N1" s="30"/>
-      <c r="O1" s="28" t="s">
+      <c r="M1" s="29" t="s">
+        <v>0</v>
+      </c>
+      <c r="N1" s="31"/>
+      <c r="O1" s="29" t="s">
         <v>5</v>
       </c>
-      <c r="P1" s="30"/>
-      <c r="Q1" s="33" t="s">
+      <c r="P1" s="31"/>
+      <c r="Q1" s="34" t="s">
         <v>79</v>
       </c>
-      <c r="R1" s="33" t="s">
+      <c r="R1" s="34" t="s">
         <v>45</v>
       </c>
-      <c r="S1" s="33" t="s">
+      <c r="S1" s="34" t="s">
         <v>84</v>
       </c>
       <c r="Y1" s="17" t="s">
@@ -27632,9 +27640,9 @@
       <c r="P2" s="8" t="s">
         <v>78</v>
       </c>
-      <c r="Q2" s="34"/>
-      <c r="R2" s="34"/>
-      <c r="S2" s="34"/>
+      <c r="Q2" s="35"/>
+      <c r="R2" s="35"/>
+      <c r="S2" s="35"/>
       <c r="Y2" s="11">
         <f>B4</f>
         <v>46091</v>
@@ -27698,7 +27706,7 @@
       </c>
       <c r="S3" s="2">
         <f ca="1">IF(COUNTIFS(D:D,"&lt;"&amp;TODAY(),J:J,"")=0,"",TODAY()-_xlfn.MINIFS(D:D,D:D,"&lt;"&amp;TODAY(),J:J,""))</f>
-        <v>38</v>
+        <v>62</v>
       </c>
       <c r="Y3" s="11">
         <f>J2</f>
@@ -27964,7 +27972,7 @@
       </c>
       <c r="B13" s="10">
         <f ca="1">IF(B11&lt;&gt;N3,(TODAY()-B12)*-1,"")</f>
-        <v>124</v>
+        <v>100</v>
       </c>
       <c r="D13" s="11"/>
       <c r="E13" s="15"/>
@@ -28480,21 +28488,21 @@
       <c r="K1" s="9" t="s">
         <v>42</v>
       </c>
-      <c r="M1" s="28" t="s">
-        <v>0</v>
-      </c>
-      <c r="N1" s="30"/>
-      <c r="O1" s="28" t="s">
+      <c r="M1" s="29" t="s">
+        <v>0</v>
+      </c>
+      <c r="N1" s="31"/>
+      <c r="O1" s="29" t="s">
         <v>5</v>
       </c>
-      <c r="P1" s="30"/>
-      <c r="Q1" s="33" t="s">
+      <c r="P1" s="31"/>
+      <c r="Q1" s="34" t="s">
         <v>79</v>
       </c>
-      <c r="R1" s="33" t="s">
+      <c r="R1" s="34" t="s">
         <v>45</v>
       </c>
-      <c r="S1" s="33" t="s">
+      <c r="S1" s="34" t="s">
         <v>84</v>
       </c>
       <c r="Y1" s="17" t="s">
@@ -28551,9 +28559,9 @@
       <c r="P2" s="8" t="s">
         <v>78</v>
       </c>
-      <c r="Q2" s="34"/>
-      <c r="R2" s="34"/>
-      <c r="S2" s="34"/>
+      <c r="Q2" s="35"/>
+      <c r="R2" s="35"/>
+      <c r="S2" s="35"/>
       <c r="Y2" s="11">
         <f>B4</f>
         <v>46073</v>
@@ -29400,21 +29408,21 @@
       <c r="K1" s="9" t="s">
         <v>42</v>
       </c>
-      <c r="M1" s="28" t="s">
-        <v>0</v>
-      </c>
-      <c r="N1" s="30"/>
-      <c r="O1" s="28" t="s">
+      <c r="M1" s="29" t="s">
+        <v>0</v>
+      </c>
+      <c r="N1" s="31"/>
+      <c r="O1" s="29" t="s">
         <v>5</v>
       </c>
-      <c r="P1" s="30"/>
-      <c r="Q1" s="33" t="s">
+      <c r="P1" s="31"/>
+      <c r="Q1" s="34" t="s">
         <v>79</v>
       </c>
-      <c r="R1" s="33" t="s">
+      <c r="R1" s="34" t="s">
         <v>45</v>
       </c>
-      <c r="S1" s="33" t="s">
+      <c r="S1" s="34" t="s">
         <v>84</v>
       </c>
       <c r="Y1" s="17" t="s">
@@ -29471,9 +29479,9 @@
       <c r="P2" s="8" t="s">
         <v>78</v>
       </c>
-      <c r="Q2" s="34"/>
-      <c r="R2" s="34"/>
-      <c r="S2" s="34"/>
+      <c r="Q2" s="35"/>
+      <c r="R2" s="35"/>
+      <c r="S2" s="35"/>
       <c r="Y2" s="11">
         <f>B4</f>
         <v>46073</v>
@@ -29803,7 +29811,7 @@
       </c>
       <c r="B13" s="10">
         <f ca="1">IF(B11&lt;&gt;N3,(TODAY()-B12)*-1,"")</f>
-        <v>105</v>
+        <v>81</v>
       </c>
       <c r="D13" s="11"/>
       <c r="E13" s="15"/>

</xml_diff>